<commit_message>
feat(facies): make p10 audit blocker-aware
</commit_message>
<xml_diff>
--- a/_pipelines/02_task_datasets/facies/_outputs/p10_model_results/track_model_metrics.xlsx
+++ b/_pipelines/02_task_datasets/facies/_outputs/p10_model_results/track_model_metrics.xlsx
@@ -421,19 +421,19 @@
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
     <col width="31" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="39" customWidth="1" min="7" max="7"/>
     <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="39" customWidth="1" min="9" max="9"/>
     <col width="48" customWidth="1" min="10" max="10"/>
     <col width="37" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
     <col width="21" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="23" customWidth="1" min="16" max="16"/>
+    <col width="33" customWidth="1" min="16" max="16"/>
     <col width="22" customWidth="1" min="17" max="17"/>
     <col width="24" customWidth="1" min="18" max="18"/>
     <col width="25" customWidth="1" min="19" max="19"/>
@@ -77386,7 +77386,7 @@
       </c>
       <c r="B642" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>Penobscot</t>
         </is>
       </c>
       <c r="C642" t="inlineStr">
@@ -77429,12 +77429,12 @@
       </c>
       <c r="K642" t="inlineStr">
         <is>
-          <t>p9_sam2_effect_macro_fold</t>
+          <t>p9_sam2_effect_locked_manifest_fold</t>
         </is>
       </c>
       <c r="L642" t="inlineStr">
         <is>
-          <t>aggregate_macro_fold</t>
+          <t>fold_0</t>
         </is>
       </c>
       <c r="M642" t="inlineStr">
@@ -77443,24 +77443,24 @@
         </is>
       </c>
       <c r="N642" t="n">
-        <v>0.0820173614809763</v>
+        <v>0.07287120819091797</v>
       </c>
       <c r="O642" t="b">
         <v>1</v>
       </c>
       <c r="P642" t="inlineStr">
         <is>
-          <t>smp_fpn_r18</t>
+          <t>smp_deeplabv3plus_r18</t>
         </is>
       </c>
       <c r="Q642" t="n">
-        <v>0.1313164220202209</v>
+        <v>0.1575457119899479</v>
       </c>
       <c r="R642" t="n">
-        <v>-0.04929906053924463</v>
+        <v>-0.08467450379902994</v>
       </c>
       <c r="S642" t="n">
-        <v>-0.3754218991106326</v>
+        <v>-0.5374599075373917</v>
       </c>
       <c r="T642" t="inlineStr">
         <is>
@@ -77469,7 +77469,7 @@
       </c>
       <c r="U642" t="inlineStr">
         <is>
-          <t>_pipelines/02_task_datasets/facies/_outputs/p9_sam2_effect/facies_f3/summary.json</t>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p9_sam2_effect/facies_penobscot/summary.json</t>
         </is>
       </c>
       <c r="V642" t="inlineStr">
@@ -77484,7 +77484,7 @@
       </c>
       <c r="X642" t="inlineStr">
         <is>
-          <t>pretrained_foundation_underperforms_locked_baseline_on_same_split</t>
+          <t>same_split_pretrained_foundation_did_not_beat_locked_baseline</t>
         </is>
       </c>
       <c r="Y642" t="inlineStr">
@@ -77494,7 +77494,7 @@
       </c>
       <c r="Z642" t="inlineStr">
         <is>
-          <t>pretrained=0.082017 random_init=0.032214; frozen test not opened</t>
+          <t>pretrained=0.072871 random_init=0.072871 baseline_fold=0.157546; no frozen test</t>
         </is>
       </c>
     </row>
@@ -77516,7 +77516,7 @@
       </c>
       <c r="D643" t="inlineStr">
         <is>
-          <t>facebook/sam2.1-hiera-base-plus</t>
+          <t>sam2.1-hiera-base-plus-random-init</t>
         </is>
       </c>
       <c r="E643" t="inlineStr">
@@ -77584,7 +77584,7 @@
       </c>
       <c r="T643" t="inlineStr">
         <is>
-          <t>non_beneficial</t>
+          <t>control</t>
         </is>
       </c>
       <c r="U643" t="inlineStr">
@@ -77636,7 +77636,7 @@
       </c>
       <c r="D644" t="inlineStr">
         <is>
-          <t>sam2.1-hiera-base-plus-random-init</t>
+          <t>facebook/sam2.1-hiera-base-plus</t>
         </is>
       </c>
       <c r="E644" t="inlineStr">
@@ -77674,7 +77674,7 @@
       </c>
       <c r="L644" t="inlineStr">
         <is>
-          <t>fold_0</t>
+          <t>fold_1</t>
         </is>
       </c>
       <c r="M644" t="inlineStr">
@@ -77683,7 +77683,7 @@
         </is>
       </c>
       <c r="N644" t="n">
-        <v>0.07287120819091797</v>
+        <v>0.09067709110802034</v>
       </c>
       <c r="O644" t="b">
         <v>1</v>
@@ -77694,17 +77694,17 @@
         </is>
       </c>
       <c r="Q644" t="n">
-        <v>0.1575457119899479</v>
+        <v>0.1341856297229407</v>
       </c>
       <c r="R644" t="n">
-        <v>-0.08467450379902994</v>
+        <v>-0.04350853861492031</v>
       </c>
       <c r="S644" t="n">
-        <v>-0.5374599075373917</v>
+        <v>-0.3242414161989955</v>
       </c>
       <c r="T644" t="inlineStr">
         <is>
-          <t>control</t>
+          <t>non_beneficial</t>
         </is>
       </c>
       <c r="U644" t="inlineStr">
@@ -77734,7 +77734,7 @@
       </c>
       <c r="Z644" t="inlineStr">
         <is>
-          <t>pretrained=0.072871 random_init=0.072871 baseline_fold=0.157546; no frozen test</t>
+          <t>pretrained=0.090677 random_init=0.088995 baseline_fold=0.134186; no frozen test</t>
         </is>
       </c>
     </row>
@@ -77756,7 +77756,7 @@
       </c>
       <c r="D645" t="inlineStr">
         <is>
-          <t>facebook/sam2.1-hiera-base-plus</t>
+          <t>sam2.1-hiera-base-plus-random-init</t>
         </is>
       </c>
       <c r="E645" t="inlineStr">
@@ -77803,7 +77803,7 @@
         </is>
       </c>
       <c r="N645" t="n">
-        <v>0.09067709110802034</v>
+        <v>0.08899497985839844</v>
       </c>
       <c r="O645" t="b">
         <v>1</v>
@@ -77817,14 +77817,14 @@
         <v>0.1341856297229407</v>
       </c>
       <c r="R645" t="n">
-        <v>-0.04350853861492031</v>
+        <v>-0.04519064986454221</v>
       </c>
       <c r="S645" t="n">
-        <v>-0.3242414161989955</v>
+        <v>-0.3367771195607865</v>
       </c>
       <c r="T645" t="inlineStr">
         <is>
-          <t>non_beneficial</t>
+          <t>control</t>
         </is>
       </c>
       <c r="U645" t="inlineStr">
@@ -77876,7 +77876,7 @@
       </c>
       <c r="D646" t="inlineStr">
         <is>
-          <t>sam2.1-hiera-base-plus-random-init</t>
+          <t>facebook/sam2.1-hiera-base-plus</t>
         </is>
       </c>
       <c r="E646" t="inlineStr">
@@ -77914,7 +77914,7 @@
       </c>
       <c r="L646" t="inlineStr">
         <is>
-          <t>fold_1</t>
+          <t>fold_2</t>
         </is>
       </c>
       <c r="M646" t="inlineStr">
@@ -77923,7 +77923,7 @@
         </is>
       </c>
       <c r="N646" t="n">
-        <v>0.08899497985839844</v>
+        <v>0.09305820824458683</v>
       </c>
       <c r="O646" t="b">
         <v>1</v>
@@ -77934,17 +77934,17 @@
         </is>
       </c>
       <c r="Q646" t="n">
-        <v>0.1341856297229407</v>
+        <v>0.1240970106393453</v>
       </c>
       <c r="R646" t="n">
-        <v>-0.04519064986454221</v>
+        <v>-0.03103880239475844</v>
       </c>
       <c r="S646" t="n">
-        <v>-0.3367771195607865</v>
+        <v>-0.2501172448461664</v>
       </c>
       <c r="T646" t="inlineStr">
         <is>
-          <t>control</t>
+          <t>non_beneficial</t>
         </is>
       </c>
       <c r="U646" t="inlineStr">
@@ -77974,7 +77974,7 @@
       </c>
       <c r="Z646" t="inlineStr">
         <is>
-          <t>pretrained=0.090677 random_init=0.088995 baseline_fold=0.134186; no frozen test</t>
+          <t>pretrained=0.093058 random_init=0.094182 baseline_fold=0.124097; no frozen test</t>
         </is>
       </c>
     </row>
@@ -77996,7 +77996,7 @@
       </c>
       <c r="D647" t="inlineStr">
         <is>
-          <t>facebook/sam2.1-hiera-base-plus</t>
+          <t>sam2.1-hiera-base-plus-random-init</t>
         </is>
       </c>
       <c r="E647" t="inlineStr">
@@ -78043,7 +78043,7 @@
         </is>
       </c>
       <c r="N647" t="n">
-        <v>0.09305820824458683</v>
+        <v>0.09418230683039444</v>
       </c>
       <c r="O647" t="b">
         <v>1</v>
@@ -78057,14 +78057,14 @@
         <v>0.1240970106393453</v>
       </c>
       <c r="R647" t="n">
-        <v>-0.03103880239475844</v>
+        <v>-0.02991470380895082</v>
       </c>
       <c r="S647" t="n">
-        <v>-0.2501172448461664</v>
+        <v>-0.2410590203166932</v>
       </c>
       <c r="T647" t="inlineStr">
         <is>
-          <t>non_beneficial</t>
+          <t>control</t>
         </is>
       </c>
       <c r="U647" t="inlineStr">
@@ -78116,7 +78116,7 @@
       </c>
       <c r="D648" t="inlineStr">
         <is>
-          <t>sam2.1-hiera-base-plus-random-init</t>
+          <t>facebook/sam2.1-hiera-base-plus</t>
         </is>
       </c>
       <c r="E648" t="inlineStr">
@@ -78154,7 +78154,7 @@
       </c>
       <c r="L648" t="inlineStr">
         <is>
-          <t>fold_2</t>
+          <t>fold_3</t>
         </is>
       </c>
       <c r="M648" t="inlineStr">
@@ -78163,7 +78163,7 @@
         </is>
       </c>
       <c r="N648" t="n">
-        <v>0.09418230683039444</v>
+        <v>0.08102512359619141</v>
       </c>
       <c r="O648" t="b">
         <v>1</v>
@@ -78174,17 +78174,17 @@
         </is>
       </c>
       <c r="Q648" t="n">
-        <v>0.1240970106393453</v>
+        <v>0.08838164651446252</v>
       </c>
       <c r="R648" t="n">
-        <v>-0.02991470380895082</v>
+        <v>-0.007356522918271116</v>
       </c>
       <c r="S648" t="n">
-        <v>-0.2410590203166932</v>
+        <v>-0.08323586636358167</v>
       </c>
       <c r="T648" t="inlineStr">
         <is>
-          <t>control</t>
+          <t>non_beneficial</t>
         </is>
       </c>
       <c r="U648" t="inlineStr">
@@ -78214,7 +78214,7 @@
       </c>
       <c r="Z648" t="inlineStr">
         <is>
-          <t>pretrained=0.093058 random_init=0.094182 baseline_fold=0.124097; no frozen test</t>
+          <t>pretrained=0.081025 random_init=0.081025 baseline_fold=0.088382; no frozen test</t>
         </is>
       </c>
     </row>
@@ -78236,7 +78236,7 @@
       </c>
       <c r="D649" t="inlineStr">
         <is>
-          <t>facebook/sam2.1-hiera-base-plus</t>
+          <t>sam2.1-hiera-base-plus-random-init</t>
         </is>
       </c>
       <c r="E649" t="inlineStr">
@@ -78304,7 +78304,7 @@
       </c>
       <c r="T649" t="inlineStr">
         <is>
-          <t>non_beneficial</t>
+          <t>control</t>
         </is>
       </c>
       <c r="U649" t="inlineStr">
@@ -78356,7 +78356,7 @@
       </c>
       <c r="D650" t="inlineStr">
         <is>
-          <t>sam2.1-hiera-base-plus-random-init</t>
+          <t>facebook/sam2.1-hiera-base-plus</t>
         </is>
       </c>
       <c r="E650" t="inlineStr">
@@ -78394,7 +78394,7 @@
       </c>
       <c r="L650" t="inlineStr">
         <is>
-          <t>fold_3</t>
+          <t>fold_4</t>
         </is>
       </c>
       <c r="M650" t="inlineStr">
@@ -78403,7 +78403,7 @@
         </is>
       </c>
       <c r="N650" t="n">
-        <v>0.08102512359619141</v>
+        <v>0.04614067077636719</v>
       </c>
       <c r="O650" t="b">
         <v>1</v>
@@ -78414,17 +78414,17 @@
         </is>
       </c>
       <c r="Q650" t="n">
-        <v>0.08838164651446252</v>
+        <v>0.1558970598677566</v>
       </c>
       <c r="R650" t="n">
-        <v>-0.007356522918271116</v>
+        <v>-0.1097563890913894</v>
       </c>
       <c r="S650" t="n">
-        <v>-0.08323586636358167</v>
+        <v>-0.7040311676467336</v>
       </c>
       <c r="T650" t="inlineStr">
         <is>
-          <t>control</t>
+          <t>non_beneficial</t>
         </is>
       </c>
       <c r="U650" t="inlineStr">
@@ -78454,7 +78454,7 @@
       </c>
       <c r="Z650" t="inlineStr">
         <is>
-          <t>pretrained=0.081025 random_init=0.081025 baseline_fold=0.088382; no frozen test</t>
+          <t>pretrained=0.046141 random_init=0.046141 baseline_fold=0.155897; no frozen test</t>
         </is>
       </c>
     </row>
@@ -78476,7 +78476,7 @@
       </c>
       <c r="D651" t="inlineStr">
         <is>
-          <t>facebook/sam2.1-hiera-base-plus</t>
+          <t>sam2.1-hiera-base-plus-random-init</t>
         </is>
       </c>
       <c r="E651" t="inlineStr">
@@ -78544,7 +78544,7 @@
       </c>
       <c r="T651" t="inlineStr">
         <is>
-          <t>non_beneficial</t>
+          <t>control</t>
         </is>
       </c>
       <c r="U651" t="inlineStr">
@@ -78586,7 +78586,7 @@
       </c>
       <c r="B652" t="inlineStr">
         <is>
-          <t>Penobscot</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="C652" t="inlineStr">
@@ -78596,7 +78596,7 @@
       </c>
       <c r="D652" t="inlineStr">
         <is>
-          <t>sam2.1-hiera-base-plus-random-init</t>
+          <t>facebook/sam2.1-hiera-base-plus+gated-residual</t>
         </is>
       </c>
       <c r="E652" t="inlineStr">
@@ -78614,27 +78614,27 @@
       </c>
       <c r="H652" t="inlineStr">
         <is>
-          <t>adapter_plus_semantic_head</t>
+          <t>gated_residual_repair_audit</t>
         </is>
       </c>
       <c r="I652" t="inlineStr">
         <is>
-          <t>fpn_projections_plus_semantic_head</t>
+          <t>base_logits_plus_gated_residual_probe</t>
         </is>
       </c>
       <c r="J652" t="inlineStr">
         <is>
-          <t>p9_sam2_effect_identity_norm</t>
+          <t>p10_sam2_repair_audit_identity_norm</t>
         </is>
       </c>
       <c r="K652" t="inlineStr">
         <is>
-          <t>p9_sam2_effect_locked_manifest_fold</t>
+          <t>p10_sam2_repair_audit_blocked</t>
         </is>
       </c>
       <c r="L652" t="inlineStr">
         <is>
-          <t>fold_4</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="M652" t="inlineStr">
@@ -78643,33 +78643,33 @@
         </is>
       </c>
       <c r="N652" t="n">
-        <v>0.04614067077636719</v>
+        <v/>
       </c>
       <c r="O652" t="b">
         <v>1</v>
       </c>
       <c r="P652" t="inlineStr">
         <is>
-          <t>smp_deeplabv3plus_r18</t>
+          <t>facebook/sam2.1-hiera-base-plus</t>
         </is>
       </c>
       <c r="Q652" t="n">
-        <v>0.1558970598677566</v>
+        <v/>
       </c>
       <c r="R652" t="n">
-        <v>-0.1097563890913894</v>
+        <v/>
       </c>
       <c r="S652" t="n">
-        <v>-0.7040311676467336</v>
+        <v>0</v>
       </c>
       <c r="T652" t="inlineStr">
         <is>
-          <t>control</t>
+          <t>data_blocked</t>
         </is>
       </c>
       <c r="U652" t="inlineStr">
         <is>
-          <t>_pipelines/02_task_datasets/facies/_outputs/p9_sam2_effect/facies_penobscot/summary.json</t>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p10_model_results/p10_sam2_repair_audit/repair_blocker.json</t>
         </is>
       </c>
       <c r="V652" t="inlineStr">
@@ -78684,7 +78684,7 @@
       </c>
       <c r="X652" t="inlineStr">
         <is>
-          <t>same_split_pretrained_foundation_did_not_beat_locked_baseline</t>
+          <t>missing_hydra_dependency_in_sam2_checkout</t>
         </is>
       </c>
       <c r="Y652" t="inlineStr">
@@ -78694,7 +78694,7 @@
       </c>
       <c r="Z652" t="inlineStr">
         <is>
-          <t>pretrained=0.046141 random_init=0.046141 baseline_fold=0.155897; no frozen test</t>
+          <t>repair probe could not execute: ModuleNotFoundError: No module named 'hydra'; checked in system python and torch-common env</t>
         </is>
       </c>
     </row>
@@ -78716,7 +78716,7 @@
       </c>
       <c r="D653" t="inlineStr">
         <is>
-          <t>facebook/sam2.1-hiera-base-plus</t>
+          <t>facebook/sam2.1-hiera-base-plus+gated-residual</t>
         </is>
       </c>
       <c r="E653" t="inlineStr">
@@ -78734,27 +78734,27 @@
       </c>
       <c r="H653" t="inlineStr">
         <is>
-          <t>adapter_plus_semantic_head</t>
+          <t>gated_residual_repair_audit</t>
         </is>
       </c>
       <c r="I653" t="inlineStr">
         <is>
-          <t>fpn_projections_plus_semantic_head</t>
+          <t>base_logits_plus_gated_residual_probe</t>
         </is>
       </c>
       <c r="J653" t="inlineStr">
         <is>
-          <t>p9_sam2_effect_identity_norm</t>
+          <t>p10_sam2_repair_audit_identity_norm</t>
         </is>
       </c>
       <c r="K653" t="inlineStr">
         <is>
-          <t>p9_sam2_effect_macro_fold</t>
+          <t>p10_sam2_repair_audit_blocked</t>
         </is>
       </c>
       <c r="L653" t="inlineStr">
         <is>
-          <t>aggregate_macro_fold</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="M653" t="inlineStr">
@@ -78763,33 +78763,33 @@
         </is>
       </c>
       <c r="N653" t="n">
-        <v>0.07675446038321675</v>
+        <v/>
       </c>
       <c r="O653" t="b">
         <v>1</v>
       </c>
       <c r="P653" t="inlineStr">
         <is>
-          <t>smp_deeplabv3plus_r18</t>
+          <t>facebook/sam2.1-hiera-base-plus</t>
         </is>
       </c>
       <c r="Q653" t="n">
-        <v>0.1320214117468906</v>
+        <v/>
       </c>
       <c r="R653" t="n">
-        <v>-0.05526695136367384</v>
+        <v/>
       </c>
       <c r="S653" t="n">
-        <v>-0.418621120865082</v>
+        <v>0</v>
       </c>
       <c r="T653" t="inlineStr">
         <is>
-          <t>non_beneficial</t>
+          <t>data_blocked</t>
         </is>
       </c>
       <c r="U653" t="inlineStr">
         <is>
-          <t>_pipelines/02_task_datasets/facies/_outputs/p9_sam2_effect/facies_penobscot/summary.json</t>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p10_model_results/p10_sam2_repair_audit/repair_blocker.json</t>
         </is>
       </c>
       <c r="V653" t="inlineStr">
@@ -78804,7 +78804,7 @@
       </c>
       <c r="X653" t="inlineStr">
         <is>
-          <t>pretrained_foundation_underperforms_locked_baseline_on_same_split</t>
+          <t>missing_hydra_dependency_in_sam2_checkout</t>
         </is>
       </c>
       <c r="Y653" t="inlineStr">
@@ -78814,7 +78814,7 @@
       </c>
       <c r="Z653" t="inlineStr">
         <is>
-          <t>pretrained=0.076754 random_init=0.076643; frozen test not opened</t>
+          <t>repair probe could not execute: ModuleNotFoundError: No module named 'hydra'; checked in system python and torch-common env</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(facies): replace false SAM2 blocker with real audit
</commit_message>
<xml_diff>
--- a/_pipelines/02_task_datasets/facies/_outputs/p10_model_results/track_model_metrics.xlsx
+++ b/_pipelines/02_task_datasets/facies/_outputs/p10_model_results/track_model_metrics.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型指标" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'模型指标'!$A$1:$Z$667</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'模型指标'!$A$1:$Z$681</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z667"/>
+  <dimension ref="A1:Z681"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -428,21 +428,21 @@
     <col width="34" customWidth="1" min="8" max="8"/>
     <col width="39" customWidth="1" min="9" max="9"/>
     <col width="48" customWidth="1" min="10" max="10"/>
-    <col width="37" customWidth="1" min="11" max="11"/>
-    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="48" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
     <col width="21" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="23" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="33" customWidth="1" min="16" max="16"/>
-    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="36" customWidth="1" min="16" max="16"/>
+    <col width="23" customWidth="1" min="17" max="17"/>
     <col width="24" customWidth="1" min="18" max="18"/>
     <col width="25" customWidth="1" min="19" max="19"/>
-    <col width="19" customWidth="1" min="20" max="20"/>
+    <col width="31" customWidth="1" min="20" max="20"/>
     <col width="48" customWidth="1" min="21" max="21"/>
     <col width="48" customWidth="1" min="22" max="22"/>
     <col width="42" customWidth="1" min="23" max="23"/>
     <col width="48" customWidth="1" min="24" max="24"/>
-    <col width="13" customWidth="1" min="25" max="25"/>
+    <col width="29" customWidth="1" min="25" max="25"/>
     <col width="48" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
@@ -78596,7 +78596,7 @@
       </c>
       <c r="D652" t="inlineStr">
         <is>
-          <t>facebook/sam2.1-hiera-base-plus+gated-residual</t>
+          <t>facebook/sam2.1-hiera-base-plus</t>
         </is>
       </c>
       <c r="E652" t="inlineStr">
@@ -78619,22 +78619,22 @@
       </c>
       <c r="I652" t="inlineStr">
         <is>
-          <t>base_logits_plus_gated_residual_probe</t>
+          <t>semantic_adapter</t>
         </is>
       </c>
       <c r="J652" t="inlineStr">
         <is>
-          <t>p10_sam2_repair_audit_identity_norm</t>
+          <t>p10_sam2_repair_audit_v1</t>
         </is>
       </c>
       <c r="K652" t="inlineStr">
         <is>
-          <t>p10_sam2_repair_audit_blocked</t>
+          <t>p10_sam2_repair_audit_dev;manifest=76a501385482bedce4e48dc44dfe5e9854b1b7aa0674fc223b3a6b42760f4614</t>
         </is>
       </c>
       <c r="L652" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>fold_0;seed_2693</t>
         </is>
       </c>
       <c r="M652" t="inlineStr">
@@ -78643,33 +78643,33 @@
         </is>
       </c>
       <c r="N652" t="n">
-        <v/>
+        <v>0.06743936319273369</v>
       </c>
       <c r="O652" t="b">
         <v>1</v>
       </c>
       <c r="P652" t="inlineStr">
         <is>
-          <t>facebook/sam2.1-hiera-base-plus</t>
+          <t>sam2.1-hiera-base-plus-random-init</t>
         </is>
       </c>
       <c r="Q652" t="n">
-        <v/>
+        <v>0.01706962783003651</v>
       </c>
       <c r="R652" t="n">
-        <v/>
+        <v>0.05036973536269719</v>
       </c>
       <c r="S652" t="n">
-        <v>0</v>
+        <v>2.950839694001077</v>
       </c>
       <c r="T652" t="inlineStr">
         <is>
-          <t>data_blocked</t>
+          <t>effect_supported_not_promoted</t>
         </is>
       </c>
       <c r="U652" t="inlineStr">
         <is>
-          <t>_pipelines/02_task_datasets/facies/_outputs/p10_model_results/p10_sam2_repair_audit/repair_blocker.json</t>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p10_sam2_repair_audit/facies_f3/summary.json</t>
         </is>
       </c>
       <c r="V652" t="inlineStr">
@@ -78684,7 +78684,7 @@
       </c>
       <c r="X652" t="inlineStr">
         <is>
-          <t>missing_hydra_dependency_in_sam2_checkout</t>
+          <t>pretraining improves the same architecture, but the adapter remains below the locked strong baseline</t>
         </is>
       </c>
       <c r="Y652" t="inlineStr">
@@ -78694,7 +78694,7 @@
       </c>
       <c r="Z652" t="inlineStr">
         <is>
-          <t>repair probe could not execute: ModuleNotFoundError: No module named 'hydra'; checked in system python and torch-common env</t>
+          <t>train_samples=32; validation_samples=16; frozen_test_accessed=False; real_pretrained_weights_loaded=True</t>
         </is>
       </c>
     </row>
@@ -78706,7 +78706,7 @@
       </c>
       <c r="B653" t="inlineStr">
         <is>
-          <t>Penobscot</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="C653" t="inlineStr">
@@ -78744,17 +78744,17 @@
       </c>
       <c r="J653" t="inlineStr">
         <is>
-          <t>p10_sam2_repair_audit_identity_norm</t>
+          <t>p10_sam2_repair_audit_v1</t>
         </is>
       </c>
       <c r="K653" t="inlineStr">
         <is>
-          <t>p10_sam2_repair_audit_blocked</t>
+          <t>p10_sam2_repair_audit_dev;manifest=76a501385482bedce4e48dc44dfe5e9854b1b7aa0674fc223b3a6b42760f4614</t>
         </is>
       </c>
       <c r="L653" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>fold_0;seed_2693</t>
         </is>
       </c>
       <c r="M653" t="inlineStr">
@@ -78763,7 +78763,7 @@
         </is>
       </c>
       <c r="N653" t="n">
-        <v/>
+        <v>0.01952300333587254</v>
       </c>
       <c r="O653" t="b">
         <v>1</v>
@@ -78774,22 +78774,22 @@
         </is>
       </c>
       <c r="Q653" t="n">
-        <v/>
+        <v>0.06743936319273369</v>
       </c>
       <c r="R653" t="n">
-        <v/>
+        <v>-0.04791635985686116</v>
       </c>
       <c r="S653" t="n">
-        <v>0</v>
+        <v>-0.7105102656429583</v>
       </c>
       <c r="T653" t="inlineStr">
         <is>
-          <t>data_blocked</t>
+          <t>non_beneficial</t>
         </is>
       </c>
       <c r="U653" t="inlineStr">
         <is>
-          <t>_pipelines/02_task_datasets/facies/_outputs/p10_model_results/p10_sam2_repair_audit/repair_blocker.json</t>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p10_sam2_repair_audit/facies_f3/summary.json</t>
         </is>
       </c>
       <c r="V653" t="inlineStr">
@@ -78804,17 +78804,17 @@
       </c>
       <c r="X653" t="inlineStr">
         <is>
-          <t>missing_hydra_dependency_in_sam2_checkout</t>
+          <t>the gated residual repair underfits and degrades the pretrained adapter on the fixed development fold</t>
         </is>
       </c>
       <c r="Y653" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>gated_residual_probe_tested</t>
         </is>
       </c>
       <c r="Z653" t="inlineStr">
         <is>
-          <t>repair probe could not execute: ModuleNotFoundError: No module named 'hydra'; checked in system python and torch-common env</t>
+          <t>train_samples=32; validation_samples=16; frozen_test_accessed=False; real_pretrained_weights_loaded=True</t>
         </is>
       </c>
     </row>
@@ -78836,12 +78836,12 @@
       </c>
       <c r="D654" t="inlineStr">
         <is>
-          <t>smp_fpn_r18</t>
+          <t>sam2.1-hiera-base-plus-random-init</t>
         </is>
       </c>
       <c r="E654" t="inlineStr">
         <is>
-          <t>SMP FPN ResNet18</t>
+          <t>SAM2.1 Hiera Base Plus</t>
         </is>
       </c>
       <c r="F654" t="b">
@@ -78849,41 +78849,41 @@
       </c>
       <c r="G654" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>image_segmentation_foundation_encoder</t>
         </is>
       </c>
       <c r="H654" t="inlineStr">
         <is>
-          <t>refit_final_holdout_confirmation</t>
+          <t>gated_residual_repair_audit</t>
         </is>
       </c>
       <c r="I654" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>semantic_adapter</t>
         </is>
       </c>
       <c r="J654" t="inlineStr">
         <is>
-          <t>9a14758fcbf9acd0ab3f8436e923e9fde347e77ce9c42961c113140a9b5407c4</t>
+          <t>p10_sam2_repair_audit_v1</t>
         </is>
       </c>
       <c r="K654" t="inlineStr">
         <is>
-          <t>p5_stage4_known_holdout</t>
+          <t>p10_sam2_repair_audit_dev;manifest=76a501385482bedce4e48dc44dfe5e9854b1b7aa0674fc223b3a6b42760f4614</t>
         </is>
       </c>
       <c r="L654" t="inlineStr">
         <is>
-          <t>refit_final</t>
+          <t>fold_0;seed_2693</t>
         </is>
       </c>
       <c r="M654" t="inlineStr">
         <is>
-          <t>accuracy</t>
+          <t>miou</t>
         </is>
       </c>
       <c r="N654" t="n">
-        <v>0.2388743196980337</v>
+        <v>0.01706962783003651</v>
       </c>
       <c r="O654" t="b">
         <v>1</v>
@@ -78894,27 +78894,27 @@
         </is>
       </c>
       <c r="Q654" t="n">
-        <v>0.2388743196980337</v>
+        <v>0.1310363943525718</v>
       </c>
       <c r="R654" t="n">
-        <v>0</v>
+        <v>-0.1139667665225353</v>
       </c>
       <c r="S654" t="n">
-        <v>0</v>
+        <v>-0.8697336880003865</v>
       </c>
       <c r="T654" t="inlineStr">
         <is>
-          <t>confirmed_holdout</t>
+          <t>control</t>
         </is>
       </c>
       <c r="U654" t="inlineStr">
         <is>
-          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage4_confirmation/facies_f3/metrics.json</t>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p10_sam2_repair_audit/facies_f3/summary.json</t>
         </is>
       </c>
       <c r="V654" t="inlineStr">
         <is>
-          <t>facies_f3/refit_final.ckpt</t>
+          <t>/mnt/data/yongan-admin-2/.cache/huggingface/hub/models--facebook--sam2.1-hiera-base-plus/blobs/a2345aede8715ab1d5d31b4a509fb160c5a4af1970f199d9054ccfb746c004c5</t>
         </is>
       </c>
       <c r="W654" t="inlineStr">
@@ -78924,7 +78924,7 @@
       </c>
       <c r="X654" t="inlineStr">
         <is>
-          <t>holdout_confirmation_after_locked_refit</t>
+          <t>same-architecture random initialization control</t>
         </is>
       </c>
       <c r="Y654" t="inlineStr">
@@ -78934,7 +78934,7 @@
       </c>
       <c r="Z654" t="inlineStr">
         <is>
-          <t>known holdout confirmed exactly once; no calibration or threshold tuning</t>
+          <t>train_samples=32; validation_samples=16; frozen_test_accessed=False; real_pretrained_weights_loaded=True</t>
         </is>
       </c>
     </row>
@@ -78961,7 +78961,7 @@
       </c>
       <c r="E655" t="inlineStr">
         <is>
-          <t>SMP FPN ResNet18</t>
+          <t>locked strong baseline</t>
         </is>
       </c>
       <c r="F655" t="b">
@@ -78974,27 +78974,27 @@
       </c>
       <c r="H655" t="inlineStr">
         <is>
-          <t>refit_final_holdout_confirmation</t>
+          <t>gated_residual_repair_audit</t>
         </is>
       </c>
       <c r="I655" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>semantic_adapter</t>
         </is>
       </c>
       <c r="J655" t="inlineStr">
         <is>
-          <t>9a14758fcbf9acd0ab3f8436e923e9fde347e77ce9c42961c113140a9b5407c4</t>
+          <t>p10_sam2_repair_audit_v1</t>
         </is>
       </c>
       <c r="K655" t="inlineStr">
         <is>
-          <t>p5_stage4_known_holdout</t>
+          <t>p10_sam2_repair_audit_dev;manifest=76a501385482bedce4e48dc44dfe5e9854b1b7aa0674fc223b3a6b42760f4614</t>
         </is>
       </c>
       <c r="L655" t="inlineStr">
         <is>
-          <t>refit_final</t>
+          <t>fold_0;seed_2693</t>
         </is>
       </c>
       <c r="M655" t="inlineStr">
@@ -79003,7 +79003,7 @@
         </is>
       </c>
       <c r="N655" t="n">
-        <v>0.1264948345532109</v>
+        <v>0.1310363943525718</v>
       </c>
       <c r="O655" t="b">
         <v>1</v>
@@ -79014,7 +79014,7 @@
         </is>
       </c>
       <c r="Q655" t="n">
-        <v>0.1264948345532109</v>
+        <v>0.1310363943525718</v>
       </c>
       <c r="R655" t="n">
         <v>0</v>
@@ -79024,19 +79024,15 @@
       </c>
       <c r="T655" t="inlineStr">
         <is>
-          <t>confirmed_holdout</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="U655" t="inlineStr">
         <is>
-          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage4_confirmation/facies_f3/metrics.json</t>
-        </is>
-      </c>
-      <c r="V655" t="inlineStr">
-        <is>
-          <t>facies_f3/refit_final.ckpt</t>
-        </is>
-      </c>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p10_sam2_repair_audit/facies_f3/summary.json</t>
+        </is>
+      </c>
+      <c r="V655" t="inlineStr"/>
       <c r="W655" t="inlineStr">
         <is>
           <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
@@ -79044,7 +79040,7 @@
       </c>
       <c r="X655" t="inlineStr">
         <is>
-          <t>holdout_confirmation_after_locked_refit</t>
+          <t>locked strong baseline on the same development samples</t>
         </is>
       </c>
       <c r="Y655" t="inlineStr">
@@ -79054,7 +79050,7 @@
       </c>
       <c r="Z655" t="inlineStr">
         <is>
-          <t>known holdout confirmed exactly once; no calibration or threshold tuning</t>
+          <t>train_samples=32; validation_samples=16; frozen_test_accessed=False; real_pretrained_weights_loaded=True</t>
         </is>
       </c>
     </row>
@@ -79076,85 +79072,85 @@
       </c>
       <c r="D656" t="inlineStr">
         <is>
-          <t>smp_fpn_r18</t>
+          <t>facebook/sam2.1-hiera-base-plus</t>
         </is>
       </c>
       <c r="E656" t="inlineStr">
         <is>
-          <t>SMP FPN ResNet18</t>
+          <t>SAM2.1 Hiera Base Plus</t>
         </is>
       </c>
       <c r="F656" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G656" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>image_segmentation_foundation_encoder</t>
         </is>
       </c>
       <c r="H656" t="inlineStr">
         <is>
-          <t>refit_final_holdout_confirmation</t>
+          <t>gated_residual_repair_audit</t>
         </is>
       </c>
       <c r="I656" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>semantic_adapter</t>
         </is>
       </c>
       <c r="J656" t="inlineStr">
         <is>
-          <t>9a14758fcbf9acd0ab3f8436e923e9fde347e77ce9c42961c113140a9b5407c4</t>
+          <t>p10_sam2_repair_audit_v1</t>
         </is>
       </c>
       <c r="K656" t="inlineStr">
         <is>
-          <t>p5_stage4_known_holdout</t>
+          <t>p10_sam2_repair_audit_dev;manifest=76a501385482bedce4e48dc44dfe5e9854b1b7aa0674fc223b3a6b42760f4614</t>
         </is>
       </c>
       <c r="L656" t="inlineStr">
         <is>
-          <t>refit_final</t>
+          <t>fold_4;seed_2697</t>
         </is>
       </c>
       <c r="M656" t="inlineStr">
         <is>
-          <t>macro_f1</t>
+          <t>miou</t>
         </is>
       </c>
       <c r="N656" t="n">
-        <v>0.2178131390049433</v>
+        <v>0.09473509513301279</v>
       </c>
       <c r="O656" t="b">
         <v>1</v>
       </c>
       <c r="P656" t="inlineStr">
         <is>
-          <t>smp_fpn_r18</t>
+          <t>sam2.1-hiera-base-plus-random-init</t>
         </is>
       </c>
       <c r="Q656" t="n">
-        <v>0.2178131390049433</v>
+        <v>0.02467325915190839</v>
       </c>
       <c r="R656" t="n">
-        <v>0</v>
+        <v>0.0700618359811044</v>
       </c>
       <c r="S656" t="n">
-        <v>0</v>
+        <v>2.839585785961534</v>
       </c>
       <c r="T656" t="inlineStr">
         <is>
-          <t>confirmed_holdout</t>
+          <t>effect_supported_not_promoted</t>
         </is>
       </c>
       <c r="U656" t="inlineStr">
         <is>
-          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage4_confirmation/facies_f3/metrics.json</t>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p10_sam2_repair_audit/facies_f3/summary.json</t>
         </is>
       </c>
       <c r="V656" t="inlineStr">
         <is>
-          <t>facies_f3/refit_final.ckpt</t>
+          <t>/mnt/data/yongan-admin-2/.cache/huggingface/hub/models--facebook--sam2.1-hiera-base-plus/blobs/a2345aede8715ab1d5d31b4a509fb160c5a4af1970f199d9054ccfb746c004c5</t>
         </is>
       </c>
       <c r="W656" t="inlineStr">
@@ -79164,7 +79160,7 @@
       </c>
       <c r="X656" t="inlineStr">
         <is>
-          <t>holdout_confirmation_after_locked_refit</t>
+          <t>pretraining improves the same architecture, but the adapter remains below the locked strong baseline</t>
         </is>
       </c>
       <c r="Y656" t="inlineStr">
@@ -79174,7 +79170,7 @@
       </c>
       <c r="Z656" t="inlineStr">
         <is>
-          <t>known holdout confirmed exactly once; no calibration or threshold tuning</t>
+          <t>train_samples=32; validation_samples=16; frozen_test_accessed=False; real_pretrained_weights_loaded=True</t>
         </is>
       </c>
     </row>
@@ -79196,85 +79192,85 @@
       </c>
       <c r="D657" t="inlineStr">
         <is>
-          <t>smp_fpn_r18</t>
+          <t>facebook/sam2.1-hiera-base-plus+gated-residual</t>
         </is>
       </c>
       <c r="E657" t="inlineStr">
         <is>
-          <t>SMP FPN ResNet18</t>
+          <t>SAM2.1 Hiera Base Plus</t>
         </is>
       </c>
       <c r="F657" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G657" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>image_segmentation_foundation_encoder</t>
         </is>
       </c>
       <c r="H657" t="inlineStr">
         <is>
-          <t>refit_final_holdout_confirmation</t>
+          <t>gated_residual_repair_audit</t>
         </is>
       </c>
       <c r="I657" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>base_logits_plus_gated_residual_probe</t>
         </is>
       </c>
       <c r="J657" t="inlineStr">
         <is>
-          <t>9a14758fcbf9acd0ab3f8436e923e9fde347e77ce9c42961c113140a9b5407c4</t>
+          <t>p10_sam2_repair_audit_v1</t>
         </is>
       </c>
       <c r="K657" t="inlineStr">
         <is>
-          <t>p5_stage4_known_holdout</t>
+          <t>p10_sam2_repair_audit_dev;manifest=76a501385482bedce4e48dc44dfe5e9854b1b7aa0674fc223b3a6b42760f4614</t>
         </is>
       </c>
       <c r="L657" t="inlineStr">
         <is>
-          <t>refit_final</t>
+          <t>fold_4;seed_2697</t>
         </is>
       </c>
       <c r="M657" t="inlineStr">
         <is>
-          <t>ece</t>
+          <t>miou</t>
         </is>
       </c>
       <c r="N657" t="n">
-        <v>0.2519504074355844</v>
+        <v>0.04385968351281433</v>
       </c>
       <c r="O657" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P657" t="inlineStr">
         <is>
-          <t>smp_fpn_r18</t>
+          <t>facebook/sam2.1-hiera-base-plus</t>
         </is>
       </c>
       <c r="Q657" t="n">
-        <v>0.2519504074355844</v>
+        <v>0.09473509513301279</v>
       </c>
       <c r="R657" t="n">
-        <v>0</v>
+        <v>-0.05087541162019846</v>
       </c>
       <c r="S657" t="n">
-        <v>0</v>
+        <v>-0.537028136708649</v>
       </c>
       <c r="T657" t="inlineStr">
         <is>
-          <t>confirmed_holdout</t>
+          <t>non_beneficial</t>
         </is>
       </c>
       <c r="U657" t="inlineStr">
         <is>
-          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage4_confirmation/facies_f3/metrics.json</t>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p10_sam2_repair_audit/facies_f3/summary.json</t>
         </is>
       </c>
       <c r="V657" t="inlineStr">
         <is>
-          <t>facies_f3/refit_final.ckpt</t>
+          <t>/mnt/data/yongan-admin-2/.cache/huggingface/hub/models--facebook--sam2.1-hiera-base-plus/blobs/a2345aede8715ab1d5d31b4a509fb160c5a4af1970f199d9054ccfb746c004c5</t>
         </is>
       </c>
       <c r="W657" t="inlineStr">
@@ -79284,17 +79280,17 @@
       </c>
       <c r="X657" t="inlineStr">
         <is>
-          <t>holdout_confirmation_after_locked_refit</t>
+          <t>the gated residual repair underfits and degrades the pretrained adapter on the fixed development fold</t>
         </is>
       </c>
       <c r="Y657" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>gated_residual_probe_tested</t>
         </is>
       </c>
       <c r="Z657" t="inlineStr">
         <is>
-          <t>known holdout confirmed exactly once; no calibration or threshold tuning</t>
+          <t>train_samples=32; validation_samples=16; frozen_test_accessed=False; real_pretrained_weights_loaded=True</t>
         </is>
       </c>
     </row>
@@ -79316,85 +79312,85 @@
       </c>
       <c r="D658" t="inlineStr">
         <is>
+          <t>sam2.1-hiera-base-plus-random-init</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>SAM2.1 Hiera Base Plus</t>
+        </is>
+      </c>
+      <c r="F658" t="b">
+        <v>0</v>
+      </c>
+      <c r="G658" t="inlineStr">
+        <is>
+          <t>image_segmentation_foundation_encoder</t>
+        </is>
+      </c>
+      <c r="H658" t="inlineStr">
+        <is>
+          <t>gated_residual_repair_audit</t>
+        </is>
+      </c>
+      <c r="I658" t="inlineStr">
+        <is>
+          <t>semantic_adapter</t>
+        </is>
+      </c>
+      <c r="J658" t="inlineStr">
+        <is>
+          <t>p10_sam2_repair_audit_v1</t>
+        </is>
+      </c>
+      <c r="K658" t="inlineStr">
+        <is>
+          <t>p10_sam2_repair_audit_dev;manifest=76a501385482bedce4e48dc44dfe5e9854b1b7aa0674fc223b3a6b42760f4614</t>
+        </is>
+      </c>
+      <c r="L658" t="inlineStr">
+        <is>
+          <t>fold_4;seed_2697</t>
+        </is>
+      </c>
+      <c r="M658" t="inlineStr">
+        <is>
+          <t>miou</t>
+        </is>
+      </c>
+      <c r="N658" t="n">
+        <v>0.02467325915190839</v>
+      </c>
+      <c r="O658" t="b">
+        <v>1</v>
+      </c>
+      <c r="P658" t="inlineStr">
+        <is>
           <t>smp_fpn_r18</t>
         </is>
       </c>
-      <c r="E658" t="inlineStr">
-        <is>
-          <t>SMP FPN ResNet18</t>
-        </is>
-      </c>
-      <c r="F658" t="b">
-        <v>0</v>
-      </c>
-      <c r="G658" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="H658" t="inlineStr">
-        <is>
-          <t>refit_final_holdout_confirmation</t>
-        </is>
-      </c>
-      <c r="I658" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="J658" t="inlineStr">
-        <is>
-          <t>9a14758fcbf9acd0ab3f8436e923e9fde347e77ce9c42961c113140a9b5407c4</t>
-        </is>
-      </c>
-      <c r="K658" t="inlineStr">
-        <is>
-          <t>p5_stage4_known_holdout</t>
-        </is>
-      </c>
-      <c r="L658" t="inlineStr">
-        <is>
-          <t>refit_final</t>
-        </is>
-      </c>
-      <c r="M658" t="inlineStr">
-        <is>
-          <t>brier</t>
-        </is>
-      </c>
-      <c r="N658" t="n">
-        <v>0.9753594398070996</v>
-      </c>
-      <c r="O658" t="b">
-        <v>0</v>
-      </c>
-      <c r="P658" t="inlineStr">
-        <is>
-          <t>smp_fpn_r18</t>
-        </is>
-      </c>
       <c r="Q658" t="n">
-        <v>0.9753594398070996</v>
+        <v>0.1130556260806936</v>
       </c>
       <c r="R658" t="n">
-        <v>0</v>
+        <v>-0.08838236692878519</v>
       </c>
       <c r="S658" t="n">
-        <v>0</v>
+        <v>-0.7817600060496076</v>
       </c>
       <c r="T658" t="inlineStr">
         <is>
-          <t>confirmed_holdout</t>
+          <t>control</t>
         </is>
       </c>
       <c r="U658" t="inlineStr">
         <is>
-          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage4_confirmation/facies_f3/metrics.json</t>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p10_sam2_repair_audit/facies_f3/summary.json</t>
         </is>
       </c>
       <c r="V658" t="inlineStr">
         <is>
-          <t>facies_f3/refit_final.ckpt</t>
+          <t>/mnt/data/yongan-admin-2/.cache/huggingface/hub/models--facebook--sam2.1-hiera-base-plus/blobs/a2345aede8715ab1d5d31b4a509fb160c5a4af1970f199d9054ccfb746c004c5</t>
         </is>
       </c>
       <c r="W658" t="inlineStr">
@@ -79404,7 +79400,7 @@
       </c>
       <c r="X658" t="inlineStr">
         <is>
-          <t>holdout_confirmation_after_locked_refit</t>
+          <t>same-architecture random initialization control</t>
         </is>
       </c>
       <c r="Y658" t="inlineStr">
@@ -79414,7 +79410,7 @@
       </c>
       <c r="Z658" t="inlineStr">
         <is>
-          <t>known holdout confirmed exactly once; no calibration or threshold tuning</t>
+          <t>train_samples=32; validation_samples=16; frozen_test_accessed=False; real_pretrained_weights_loaded=True</t>
         </is>
       </c>
     </row>
@@ -79441,7 +79437,7 @@
       </c>
       <c r="E659" t="inlineStr">
         <is>
-          <t>SMP FPN ResNet18</t>
+          <t>locked strong baseline</t>
         </is>
       </c>
       <c r="F659" t="b">
@@ -79454,39 +79450,39 @@
       </c>
       <c r="H659" t="inlineStr">
         <is>
-          <t>refit_final_holdout_confirmation</t>
+          <t>gated_residual_repair_audit</t>
         </is>
       </c>
       <c r="I659" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>semantic_adapter</t>
         </is>
       </c>
       <c r="J659" t="inlineStr">
         <is>
-          <t>9a14758fcbf9acd0ab3f8436e923e9fde347e77ce9c42961c113140a9b5407c4</t>
+          <t>p10_sam2_repair_audit_v1</t>
         </is>
       </c>
       <c r="K659" t="inlineStr">
         <is>
-          <t>p5_stage4_known_holdout</t>
+          <t>p10_sam2_repair_audit_dev;manifest=76a501385482bedce4e48dc44dfe5e9854b1b7aa0674fc223b3a6b42760f4614</t>
         </is>
       </c>
       <c r="L659" t="inlineStr">
         <is>
-          <t>refit_final</t>
+          <t>fold_4;seed_2697</t>
         </is>
       </c>
       <c r="M659" t="inlineStr">
         <is>
-          <t>nll</t>
+          <t>miou</t>
         </is>
       </c>
       <c r="N659" t="n">
-        <v>2.874396510552791</v>
+        <v>0.1130556260806936</v>
       </c>
       <c r="O659" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P659" t="inlineStr">
         <is>
@@ -79494,7 +79490,7 @@
         </is>
       </c>
       <c r="Q659" t="n">
-        <v>2.874396510552791</v>
+        <v>0.1130556260806936</v>
       </c>
       <c r="R659" t="n">
         <v>0</v>
@@ -79504,19 +79500,15 @@
       </c>
       <c r="T659" t="inlineStr">
         <is>
-          <t>confirmed_holdout</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="U659" t="inlineStr">
         <is>
-          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage4_confirmation/facies_f3/metrics.json</t>
-        </is>
-      </c>
-      <c r="V659" t="inlineStr">
-        <is>
-          <t>facies_f3/refit_final.ckpt</t>
-        </is>
-      </c>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p10_sam2_repair_audit/facies_f3/summary.json</t>
+        </is>
+      </c>
+      <c r="V659" t="inlineStr"/>
       <c r="W659" t="inlineStr">
         <is>
           <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
@@ -79524,7 +79516,7 @@
       </c>
       <c r="X659" t="inlineStr">
         <is>
-          <t>holdout_confirmation_after_locked_refit</t>
+          <t>locked strong baseline on the same development samples</t>
         </is>
       </c>
       <c r="Y659" t="inlineStr">
@@ -79534,7 +79526,7 @@
       </c>
       <c r="Z659" t="inlineStr">
         <is>
-          <t>known holdout confirmed exactly once; no calibration or threshold tuning</t>
+          <t>train_samples=32; validation_samples=16; frozen_test_accessed=False; real_pretrained_weights_loaded=True</t>
         </is>
       </c>
     </row>
@@ -79556,85 +79548,85 @@
       </c>
       <c r="D660" t="inlineStr">
         <is>
-          <t>smp_deeplabv3plus_r18</t>
+          <t>facebook/sam2.1-hiera-base-plus</t>
         </is>
       </c>
       <c r="E660" t="inlineStr">
         <is>
-          <t>SMP DeepLabV3+ ResNet18</t>
+          <t>SAM2.1 Hiera Base Plus</t>
         </is>
       </c>
       <c r="F660" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G660" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>image_segmentation_foundation_encoder</t>
         </is>
       </c>
       <c r="H660" t="inlineStr">
         <is>
-          <t>refit_final_holdout_confirmation</t>
+          <t>gated_residual_repair_audit</t>
         </is>
       </c>
       <c r="I660" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>semantic_adapter</t>
         </is>
       </c>
       <c r="J660" t="inlineStr">
         <is>
-          <t>399a258d1fdc8c396891f2735d7ee95d9d467bf0f43f209e0a0a9213266331e9</t>
+          <t>p10_sam2_repair_audit_v1</t>
         </is>
       </c>
       <c r="K660" t="inlineStr">
         <is>
-          <t>p5_stage4_known_holdout</t>
+          <t>p10_sam2_repair_audit_dev;manifest=3440bbbd415158e41c6f0ed14513208fc77075c108716f9f6593ff0847382c81</t>
         </is>
       </c>
       <c r="L660" t="inlineStr">
         <is>
-          <t>refit_final</t>
+          <t>fold_0;seed_2693</t>
         </is>
       </c>
       <c r="M660" t="inlineStr">
         <is>
-          <t>accuracy</t>
+          <t>miou</t>
         </is>
       </c>
       <c r="N660" t="n">
-        <v>0.5285719215618407</v>
+        <v>0.07287120819091797</v>
       </c>
       <c r="O660" t="b">
         <v>1</v>
       </c>
       <c r="P660" t="inlineStr">
         <is>
-          <t>smp_deeplabv3plus_r18</t>
+          <t>sam2.1-hiera-base-plus-random-init</t>
         </is>
       </c>
       <c r="Q660" t="n">
-        <v>0.5285719215618407</v>
+        <v>0.001154828957663275</v>
       </c>
       <c r="R660" t="n">
-        <v>0</v>
+        <v>0.07171637923325469</v>
       </c>
       <c r="S660" t="n">
-        <v>0</v>
+        <v>62.10129972699016</v>
       </c>
       <c r="T660" t="inlineStr">
         <is>
-          <t>confirmed_holdout</t>
+          <t>effect_supported_not_promoted</t>
         </is>
       </c>
       <c r="U660" t="inlineStr">
         <is>
-          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage4_confirmation/facies_penobscot/metrics.json</t>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p10_sam2_repair_audit/facies_penobscot/summary.json</t>
         </is>
       </c>
       <c r="V660" t="inlineStr">
         <is>
-          <t>facies_penobscot/refit_final.ckpt</t>
+          <t>/mnt/data/yongan-admin-2/.cache/huggingface/hub/models--facebook--sam2.1-hiera-base-plus/blobs/a2345aede8715ab1d5d31b4a509fb160c5a4af1970f199d9054ccfb746c004c5</t>
         </is>
       </c>
       <c r="W660" t="inlineStr">
@@ -79644,7 +79636,7 @@
       </c>
       <c r="X660" t="inlineStr">
         <is>
-          <t>holdout_confirmation_after_locked_refit</t>
+          <t>pretraining improves the same architecture, but the adapter remains below the locked strong baseline</t>
         </is>
       </c>
       <c r="Y660" t="inlineStr">
@@ -79654,7 +79646,7 @@
       </c>
       <c r="Z660" t="inlineStr">
         <is>
-          <t>known holdout confirmed exactly once; no calibration or threshold tuning</t>
+          <t>train_samples=32; validation_samples=16; frozen_test_accessed=False; real_pretrained_weights_loaded=True</t>
         </is>
       </c>
     </row>
@@ -79676,45 +79668,45 @@
       </c>
       <c r="D661" t="inlineStr">
         <is>
-          <t>smp_deeplabv3plus_r18</t>
+          <t>facebook/sam2.1-hiera-base-plus+gated-residual</t>
         </is>
       </c>
       <c r="E661" t="inlineStr">
         <is>
-          <t>SMP DeepLabV3+ ResNet18</t>
+          <t>SAM2.1 Hiera Base Plus</t>
         </is>
       </c>
       <c r="F661" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G661" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>image_segmentation_foundation_encoder</t>
         </is>
       </c>
       <c r="H661" t="inlineStr">
         <is>
-          <t>refit_final_holdout_confirmation</t>
+          <t>gated_residual_repair_audit</t>
         </is>
       </c>
       <c r="I661" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>base_logits_plus_gated_residual_probe</t>
         </is>
       </c>
       <c r="J661" t="inlineStr">
         <is>
-          <t>399a258d1fdc8c396891f2735d7ee95d9d467bf0f43f209e0a0a9213266331e9</t>
+          <t>p10_sam2_repair_audit_v1</t>
         </is>
       </c>
       <c r="K661" t="inlineStr">
         <is>
-          <t>p5_stage4_known_holdout</t>
+          <t>p10_sam2_repair_audit_dev;manifest=3440bbbd415158e41c6f0ed14513208fc77075c108716f9f6593ff0847382c81</t>
         </is>
       </c>
       <c r="L661" t="inlineStr">
         <is>
-          <t>refit_final</t>
+          <t>fold_0;seed_2693</t>
         </is>
       </c>
       <c r="M661" t="inlineStr">
@@ -79723,38 +79715,38 @@
         </is>
       </c>
       <c r="N661" t="n">
-        <v>0.125379989161776</v>
+        <v>0.01482651735997908</v>
       </c>
       <c r="O661" t="b">
         <v>1</v>
       </c>
       <c r="P661" t="inlineStr">
         <is>
-          <t>smp_deeplabv3plus_r18</t>
+          <t>facebook/sam2.1-hiera-base-plus</t>
         </is>
       </c>
       <c r="Q661" t="n">
-        <v>0.125379989161776</v>
+        <v>0.07287120819091797</v>
       </c>
       <c r="R661" t="n">
-        <v>0</v>
+        <v>-0.05804469083093888</v>
       </c>
       <c r="S661" t="n">
-        <v>0</v>
+        <v>-0.7965380603936942</v>
       </c>
       <c r="T661" t="inlineStr">
         <is>
-          <t>confirmed_holdout</t>
+          <t>non_beneficial</t>
         </is>
       </c>
       <c r="U661" t="inlineStr">
         <is>
-          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage4_confirmation/facies_penobscot/metrics.json</t>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p10_sam2_repair_audit/facies_penobscot/summary.json</t>
         </is>
       </c>
       <c r="V661" t="inlineStr">
         <is>
-          <t>facies_penobscot/refit_final.ckpt</t>
+          <t>/mnt/data/yongan-admin-2/.cache/huggingface/hub/models--facebook--sam2.1-hiera-base-plus/blobs/a2345aede8715ab1d5d31b4a509fb160c5a4af1970f199d9054ccfb746c004c5</t>
         </is>
       </c>
       <c r="W661" t="inlineStr">
@@ -79764,17 +79756,17 @@
       </c>
       <c r="X661" t="inlineStr">
         <is>
-          <t>holdout_confirmation_after_locked_refit</t>
+          <t>the gated residual repair underfits and degrades the pretrained adapter on the fixed development fold</t>
         </is>
       </c>
       <c r="Y661" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>gated_residual_probe_tested</t>
         </is>
       </c>
       <c r="Z661" t="inlineStr">
         <is>
-          <t>known holdout confirmed exactly once; no calibration or threshold tuning</t>
+          <t>train_samples=32; validation_samples=16; frozen_test_accessed=False; real_pretrained_weights_loaded=True</t>
         </is>
       </c>
     </row>
@@ -79796,12 +79788,12 @@
       </c>
       <c r="D662" t="inlineStr">
         <is>
-          <t>smp_deeplabv3plus_r18</t>
+          <t>sam2.1-hiera-base-plus-random-init</t>
         </is>
       </c>
       <c r="E662" t="inlineStr">
         <is>
-          <t>SMP DeepLabV3+ ResNet18</t>
+          <t>SAM2.1 Hiera Base Plus</t>
         </is>
       </c>
       <c r="F662" t="b">
@@ -79809,41 +79801,41 @@
       </c>
       <c r="G662" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>image_segmentation_foundation_encoder</t>
         </is>
       </c>
       <c r="H662" t="inlineStr">
         <is>
-          <t>refit_final_holdout_confirmation</t>
+          <t>gated_residual_repair_audit</t>
         </is>
       </c>
       <c r="I662" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>semantic_adapter</t>
         </is>
       </c>
       <c r="J662" t="inlineStr">
         <is>
-          <t>399a258d1fdc8c396891f2735d7ee95d9d467bf0f43f209e0a0a9213266331e9</t>
+          <t>p10_sam2_repair_audit_v1</t>
         </is>
       </c>
       <c r="K662" t="inlineStr">
         <is>
-          <t>p5_stage4_known_holdout</t>
+          <t>p10_sam2_repair_audit_dev;manifest=3440bbbd415158e41c6f0ed14513208fc77075c108716f9f6593ff0847382c81</t>
         </is>
       </c>
       <c r="L662" t="inlineStr">
         <is>
-          <t>refit_final</t>
+          <t>fold_0;seed_2693</t>
         </is>
       </c>
       <c r="M662" t="inlineStr">
         <is>
-          <t>macro_f1</t>
+          <t>miou</t>
         </is>
       </c>
       <c r="N662" t="n">
-        <v>0.1709165211603197</v>
+        <v>0.001154828957663275</v>
       </c>
       <c r="O662" t="b">
         <v>1</v>
@@ -79854,27 +79846,27 @@
         </is>
       </c>
       <c r="Q662" t="n">
-        <v>0.1709165211603197</v>
+        <v>0.1575457119899479</v>
       </c>
       <c r="R662" t="n">
-        <v>0</v>
+        <v>-0.1563908830322846</v>
       </c>
       <c r="S662" t="n">
-        <v>0</v>
+        <v>-0.9926698801060548</v>
       </c>
       <c r="T662" t="inlineStr">
         <is>
-          <t>confirmed_holdout</t>
+          <t>control</t>
         </is>
       </c>
       <c r="U662" t="inlineStr">
         <is>
-          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage4_confirmation/facies_penobscot/metrics.json</t>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p10_sam2_repair_audit/facies_penobscot/summary.json</t>
         </is>
       </c>
       <c r="V662" t="inlineStr">
         <is>
-          <t>facies_penobscot/refit_final.ckpt</t>
+          <t>/mnt/data/yongan-admin-2/.cache/huggingface/hub/models--facebook--sam2.1-hiera-base-plus/blobs/a2345aede8715ab1d5d31b4a509fb160c5a4af1970f199d9054ccfb746c004c5</t>
         </is>
       </c>
       <c r="W662" t="inlineStr">
@@ -79884,7 +79876,7 @@
       </c>
       <c r="X662" t="inlineStr">
         <is>
-          <t>holdout_confirmation_after_locked_refit</t>
+          <t>same-architecture random initialization control</t>
         </is>
       </c>
       <c r="Y662" t="inlineStr">
@@ -79894,7 +79886,7 @@
       </c>
       <c r="Z662" t="inlineStr">
         <is>
-          <t>known holdout confirmed exactly once; no calibration or threshold tuning</t>
+          <t>train_samples=32; validation_samples=16; frozen_test_accessed=False; real_pretrained_weights_loaded=True</t>
         </is>
       </c>
     </row>
@@ -79921,7 +79913,7 @@
       </c>
       <c r="E663" t="inlineStr">
         <is>
-          <t>SMP DeepLabV3+ ResNet18</t>
+          <t>locked strong baseline</t>
         </is>
       </c>
       <c r="F663" t="b">
@@ -79934,39 +79926,39 @@
       </c>
       <c r="H663" t="inlineStr">
         <is>
-          <t>refit_final_holdout_confirmation</t>
+          <t>gated_residual_repair_audit</t>
         </is>
       </c>
       <c r="I663" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>semantic_adapter</t>
         </is>
       </c>
       <c r="J663" t="inlineStr">
         <is>
-          <t>399a258d1fdc8c396891f2735d7ee95d9d467bf0f43f209e0a0a9213266331e9</t>
+          <t>p10_sam2_repair_audit_v1</t>
         </is>
       </c>
       <c r="K663" t="inlineStr">
         <is>
-          <t>p5_stage4_known_holdout</t>
+          <t>p10_sam2_repair_audit_dev;manifest=3440bbbd415158e41c6f0ed14513208fc77075c108716f9f6593ff0847382c81</t>
         </is>
       </c>
       <c r="L663" t="inlineStr">
         <is>
-          <t>refit_final</t>
+          <t>fold_0;seed_2693</t>
         </is>
       </c>
       <c r="M663" t="inlineStr">
         <is>
-          <t>ece</t>
+          <t>miou</t>
         </is>
       </c>
       <c r="N663" t="n">
-        <v>0.2939335861584093</v>
+        <v>0.1575457119899479</v>
       </c>
       <c r="O663" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P663" t="inlineStr">
         <is>
@@ -79974,7 +79966,7 @@
         </is>
       </c>
       <c r="Q663" t="n">
-        <v>0.2939335861584093</v>
+        <v>0.1575457119899479</v>
       </c>
       <c r="R663" t="n">
         <v>0</v>
@@ -79984,19 +79976,15 @@
       </c>
       <c r="T663" t="inlineStr">
         <is>
-          <t>confirmed_holdout</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="U663" t="inlineStr">
         <is>
-          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage4_confirmation/facies_penobscot/metrics.json</t>
-        </is>
-      </c>
-      <c r="V663" t="inlineStr">
-        <is>
-          <t>facies_penobscot/refit_final.ckpt</t>
-        </is>
-      </c>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p10_sam2_repair_audit/facies_penobscot/summary.json</t>
+        </is>
+      </c>
+      <c r="V663" t="inlineStr"/>
       <c r="W663" t="inlineStr">
         <is>
           <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
@@ -80004,7 +79992,7 @@
       </c>
       <c r="X663" t="inlineStr">
         <is>
-          <t>holdout_confirmation_after_locked_refit</t>
+          <t>locked strong baseline on the same development samples</t>
         </is>
       </c>
       <c r="Y663" t="inlineStr">
@@ -80014,7 +80002,7 @@
       </c>
       <c r="Z663" t="inlineStr">
         <is>
-          <t>known holdout confirmed exactly once; no calibration or threshold tuning</t>
+          <t>train_samples=32; validation_samples=16; frozen_test_accessed=False; real_pretrained_weights_loaded=True</t>
         </is>
       </c>
     </row>
@@ -80036,85 +80024,85 @@
       </c>
       <c r="D664" t="inlineStr">
         <is>
-          <t>smp_deeplabv3plus_r18</t>
+          <t>facebook/sam2.1-hiera-base-plus</t>
         </is>
       </c>
       <c r="E664" t="inlineStr">
         <is>
-          <t>SMP DeepLabV3+ ResNet18</t>
+          <t>SAM2.1 Hiera Base Plus</t>
         </is>
       </c>
       <c r="F664" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G664" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>image_segmentation_foundation_encoder</t>
         </is>
       </c>
       <c r="H664" t="inlineStr">
         <is>
-          <t>refit_final_holdout_confirmation</t>
+          <t>gated_residual_repair_audit</t>
         </is>
       </c>
       <c r="I664" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>semantic_adapter</t>
         </is>
       </c>
       <c r="J664" t="inlineStr">
         <is>
-          <t>399a258d1fdc8c396891f2735d7ee95d9d467bf0f43f209e0a0a9213266331e9</t>
+          <t>p10_sam2_repair_audit_v1</t>
         </is>
       </c>
       <c r="K664" t="inlineStr">
         <is>
-          <t>p5_stage4_known_holdout</t>
+          <t>p10_sam2_repair_audit_dev;manifest=3440bbbd415158e41c6f0ed14513208fc77075c108716f9f6593ff0847382c81</t>
         </is>
       </c>
       <c r="L664" t="inlineStr">
         <is>
-          <t>refit_final</t>
+          <t>fold_4;seed_2697</t>
         </is>
       </c>
       <c r="M664" t="inlineStr">
         <is>
-          <t>brier</t>
+          <t>miou</t>
         </is>
       </c>
       <c r="N664" t="n">
-        <v>0.7475083526250967</v>
+        <v>0.04614067077636719</v>
       </c>
       <c r="O664" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P664" t="inlineStr">
         <is>
-          <t>smp_deeplabv3plus_r18</t>
+          <t>sam2.1-hiera-base-plus-random-init</t>
         </is>
       </c>
       <c r="Q664" t="n">
-        <v>0.7475083526250967</v>
+        <v>0.01768815661407325</v>
       </c>
       <c r="R664" t="n">
-        <v>0</v>
+        <v>0.02845251416229394</v>
       </c>
       <c r="S664" t="n">
-        <v>0</v>
+        <v>1.608562994046323</v>
       </c>
       <c r="T664" t="inlineStr">
         <is>
-          <t>confirmed_holdout</t>
+          <t>effect_supported_not_promoted</t>
         </is>
       </c>
       <c r="U664" t="inlineStr">
         <is>
-          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage4_confirmation/facies_penobscot/metrics.json</t>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p10_sam2_repair_audit/facies_penobscot/summary.json</t>
         </is>
       </c>
       <c r="V664" t="inlineStr">
         <is>
-          <t>facies_penobscot/refit_final.ckpt</t>
+          <t>/mnt/data/yongan-admin-2/.cache/huggingface/hub/models--facebook--sam2.1-hiera-base-plus/blobs/a2345aede8715ab1d5d31b4a509fb160c5a4af1970f199d9054ccfb746c004c5</t>
         </is>
       </c>
       <c r="W664" t="inlineStr">
@@ -80124,7 +80112,7 @@
       </c>
       <c r="X664" t="inlineStr">
         <is>
-          <t>holdout_confirmation_after_locked_refit</t>
+          <t>pretraining improves the same architecture, but the adapter remains below the locked strong baseline</t>
         </is>
       </c>
       <c r="Y664" t="inlineStr">
@@ -80134,7 +80122,7 @@
       </c>
       <c r="Z664" t="inlineStr">
         <is>
-          <t>known holdout confirmed exactly once; no calibration or threshold tuning</t>
+          <t>train_samples=32; validation_samples=16; frozen_test_accessed=False; real_pretrained_weights_loaded=True</t>
         </is>
       </c>
     </row>
@@ -80156,85 +80144,85 @@
       </c>
       <c r="D665" t="inlineStr">
         <is>
-          <t>smp_deeplabv3plus_r18</t>
+          <t>facebook/sam2.1-hiera-base-plus+gated-residual</t>
         </is>
       </c>
       <c r="E665" t="inlineStr">
         <is>
-          <t>SMP DeepLabV3+ ResNet18</t>
+          <t>SAM2.1 Hiera Base Plus</t>
         </is>
       </c>
       <c r="F665" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G665" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>image_segmentation_foundation_encoder</t>
         </is>
       </c>
       <c r="H665" t="inlineStr">
         <is>
-          <t>refit_final_holdout_confirmation</t>
+          <t>gated_residual_repair_audit</t>
         </is>
       </c>
       <c r="I665" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>base_logits_plus_gated_residual_probe</t>
         </is>
       </c>
       <c r="J665" t="inlineStr">
         <is>
-          <t>399a258d1fdc8c396891f2735d7ee95d9d467bf0f43f209e0a0a9213266331e9</t>
+          <t>p10_sam2_repair_audit_v1</t>
         </is>
       </c>
       <c r="K665" t="inlineStr">
         <is>
-          <t>p5_stage4_known_holdout</t>
+          <t>p10_sam2_repair_audit_dev;manifest=3440bbbd415158e41c6f0ed14513208fc77075c108716f9f6593ff0847382c81</t>
         </is>
       </c>
       <c r="L665" t="inlineStr">
         <is>
-          <t>refit_final</t>
+          <t>fold_4;seed_2697</t>
         </is>
       </c>
       <c r="M665" t="inlineStr">
         <is>
-          <t>nll</t>
+          <t>miou</t>
         </is>
       </c>
       <c r="N665" t="n">
-        <v>1.879265954669352</v>
+        <v>0.03663988665881721</v>
       </c>
       <c r="O665" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P665" t="inlineStr">
         <is>
-          <t>smp_deeplabv3plus_r18</t>
+          <t>facebook/sam2.1-hiera-base-plus</t>
         </is>
       </c>
       <c r="Q665" t="n">
-        <v>1.879265954669352</v>
+        <v>0.04614067077636719</v>
       </c>
       <c r="R665" t="n">
-        <v>0</v>
+        <v>-0.009500784117549982</v>
       </c>
       <c r="S665" t="n">
-        <v>0</v>
+        <v>-0.2059091027002623</v>
       </c>
       <c r="T665" t="inlineStr">
         <is>
-          <t>confirmed_holdout</t>
+          <t>non_beneficial</t>
         </is>
       </c>
       <c r="U665" t="inlineStr">
         <is>
-          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage4_confirmation/facies_penobscot/metrics.json</t>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p10_sam2_repair_audit/facies_penobscot/summary.json</t>
         </is>
       </c>
       <c r="V665" t="inlineStr">
         <is>
-          <t>facies_penobscot/refit_final.ckpt</t>
+          <t>/mnt/data/yongan-admin-2/.cache/huggingface/hub/models--facebook--sam2.1-hiera-base-plus/blobs/a2345aede8715ab1d5d31b4a509fb160c5a4af1970f199d9054ccfb746c004c5</t>
         </is>
       </c>
       <c r="W665" t="inlineStr">
@@ -80244,17 +80232,17 @@
       </c>
       <c r="X665" t="inlineStr">
         <is>
-          <t>holdout_confirmation_after_locked_refit</t>
+          <t>the gated residual repair underfits and degrades the pretrained adapter on the fixed development fold</t>
         </is>
       </c>
       <c r="Y665" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>gated_residual_probe_tested</t>
         </is>
       </c>
       <c r="Z665" t="inlineStr">
         <is>
-          <t>known holdout confirmed exactly once; no calibration or threshold tuning</t>
+          <t>train_samples=32; validation_samples=16; frozen_test_accessed=False; real_pretrained_weights_loaded=True</t>
         </is>
       </c>
     </row>
@@ -80266,7 +80254,7 @@
       </c>
       <c r="B666" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>Penobscot</t>
         </is>
       </c>
       <c r="C666" t="inlineStr">
@@ -80276,12 +80264,12 @@
       </c>
       <c r="D666" t="inlineStr">
         <is>
-          <t>smp_fpn_r18</t>
+          <t>sam2.1-hiera-base-plus-random-init</t>
         </is>
       </c>
       <c r="E666" t="inlineStr">
         <is>
-          <t>smp fpn r18</t>
+          <t>SAM2.1 Hiera Base Plus</t>
         </is>
       </c>
       <c r="F666" t="b">
@@ -80289,32 +80277,32 @@
       </c>
       <c r="G666" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>image_segmentation_foundation_encoder</t>
         </is>
       </c>
       <c r="H666" t="inlineStr">
         <is>
-          <t>stage3_oof_leaderboard</t>
+          <t>gated_residual_repair_audit</t>
         </is>
       </c>
       <c r="I666" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>semantic_adapter</t>
         </is>
       </c>
       <c r="J666" t="inlineStr">
         <is>
-          <t>d67e14ff951b63551948bd0bf3902ad140672a875e911ad849ba4adae22ac294</t>
+          <t>p10_sam2_repair_audit_v1</t>
         </is>
       </c>
       <c r="K666" t="inlineStr">
         <is>
-          <t>p5_stage3_oof_aggregate</t>
+          <t>p10_sam2_repair_audit_dev;manifest=3440bbbd415158e41c6f0ed14513208fc77075c108716f9f6593ff0847382c81</t>
         </is>
       </c>
       <c r="L666" t="inlineStr">
         <is>
-          <t>aggregate_oof</t>
+          <t>fold_4;seed_2697</t>
         </is>
       </c>
       <c r="M666" t="inlineStr">
@@ -80323,36 +80311,40 @@
         </is>
       </c>
       <c r="N666" t="n">
-        <v>0.1313164220202209</v>
+        <v>0.01768815661407325</v>
       </c>
       <c r="O666" t="b">
         <v>1</v>
       </c>
       <c r="P666" t="inlineStr">
         <is>
-          <t>smp_fpn_r18</t>
+          <t>smp_deeplabv3plus_r18</t>
         </is>
       </c>
       <c r="Q666" t="n">
-        <v>0.1313164220202209</v>
+        <v>0.1558970598677566</v>
       </c>
       <c r="R666" t="n">
-        <v>0</v>
+        <v>-0.1382089032536833</v>
       </c>
       <c r="S666" t="n">
-        <v>0</v>
+        <v>-0.8865395112064484</v>
       </c>
       <c r="T666" t="inlineStr">
         <is>
-          <t>ranked</t>
+          <t>control</t>
         </is>
       </c>
       <c r="U666" t="inlineStr">
         <is>
-          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage3/facies_f3_scratch_leaderboard.json</t>
-        </is>
-      </c>
-      <c r="V666" t="inlineStr"/>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p10_sam2_repair_audit/facies_penobscot/summary.json</t>
+        </is>
+      </c>
+      <c r="V666" t="inlineStr">
+        <is>
+          <t>/mnt/data/yongan-admin-2/.cache/huggingface/hub/models--facebook--sam2.1-hiera-base-plus/blobs/a2345aede8715ab1d5d31b4a509fb160c5a4af1970f199d9054ccfb746c004c5</t>
+        </is>
+      </c>
       <c r="W666" t="inlineStr">
         <is>
           <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
@@ -80360,7 +80352,7 @@
       </c>
       <c r="X666" t="inlineStr">
         <is>
-          <t>current_locked_baseline_reference</t>
+          <t>same-architecture random initialization control</t>
         </is>
       </c>
       <c r="Y666" t="inlineStr">
@@ -80370,7 +80362,7 @@
       </c>
       <c r="Z666" t="inlineStr">
         <is>
-          <t>top-of-board locked baseline from frozen stage-3 leaderboard</t>
+          <t>train_samples=32; validation_samples=16; frozen_test_accessed=False; real_pretrained_weights_loaded=True</t>
         </is>
       </c>
     </row>
@@ -80397,7 +80389,7 @@
       </c>
       <c r="E667" t="inlineStr">
         <is>
-          <t>smp deeplabv3plus r18</t>
+          <t>locked strong baseline</t>
         </is>
       </c>
       <c r="F667" t="b">
@@ -80410,27 +80402,27 @@
       </c>
       <c r="H667" t="inlineStr">
         <is>
-          <t>stage3_oof_leaderboard</t>
+          <t>gated_residual_repair_audit</t>
         </is>
       </c>
       <c r="I667" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>semantic_adapter</t>
         </is>
       </c>
       <c r="J667" t="inlineStr">
         <is>
-          <t>d67e14ff951b63551948bd0bf3902ad140672a875e911ad849ba4adae22ac294</t>
+          <t>p10_sam2_repair_audit_v1</t>
         </is>
       </c>
       <c r="K667" t="inlineStr">
         <is>
-          <t>p5_stage3_oof_aggregate</t>
+          <t>p10_sam2_repair_audit_dev;manifest=3440bbbd415158e41c6f0ed14513208fc77075c108716f9f6593ff0847382c81</t>
         </is>
       </c>
       <c r="L667" t="inlineStr">
         <is>
-          <t>aggregate_oof</t>
+          <t>fold_4;seed_2697</t>
         </is>
       </c>
       <c r="M667" t="inlineStr">
@@ -80439,7 +80431,7 @@
         </is>
       </c>
       <c r="N667" t="n">
-        <v>0.1320214117468906</v>
+        <v>0.1558970598677566</v>
       </c>
       <c r="O667" t="b">
         <v>1</v>
@@ -80450,7 +80442,7 @@
         </is>
       </c>
       <c r="Q667" t="n">
-        <v>0.1320214117468906</v>
+        <v>0.1558970598677566</v>
       </c>
       <c r="R667" t="n">
         <v>0</v>
@@ -80460,12 +80452,12 @@
       </c>
       <c r="T667" t="inlineStr">
         <is>
-          <t>ranked</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="U667" t="inlineStr">
         <is>
-          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage3/facies_penobscot_scratch_leaderboard.json</t>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p10_sam2_repair_audit/facies_penobscot/summary.json</t>
         </is>
       </c>
       <c r="V667" t="inlineStr"/>
@@ -80476,22 +80468,1694 @@
       </c>
       <c r="X667" t="inlineStr">
         <is>
+          <t>locked strong baseline on the same development samples</t>
+        </is>
+      </c>
+      <c r="Y667" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z667" t="inlineStr">
+        <is>
+          <t>train_samples=32; validation_samples=16; frozen_test_accessed=False; real_pretrained_weights_loaded=True</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>facies</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>segmentation_2d</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>smp_fpn_r18</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>SMP FPN ResNet18</t>
+        </is>
+      </c>
+      <c r="F668" t="b">
+        <v>0</v>
+      </c>
+      <c r="G668" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="H668" t="inlineStr">
+        <is>
+          <t>refit_final_holdout_confirmation</t>
+        </is>
+      </c>
+      <c r="I668" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J668" t="inlineStr">
+        <is>
+          <t>9a14758fcbf9acd0ab3f8436e923e9fde347e77ce9c42961c113140a9b5407c4</t>
+        </is>
+      </c>
+      <c r="K668" t="inlineStr">
+        <is>
+          <t>p5_stage4_known_holdout</t>
+        </is>
+      </c>
+      <c r="L668" t="inlineStr">
+        <is>
+          <t>refit_final</t>
+        </is>
+      </c>
+      <c r="M668" t="inlineStr">
+        <is>
+          <t>accuracy</t>
+        </is>
+      </c>
+      <c r="N668" t="n">
+        <v>0.2388743196980337</v>
+      </c>
+      <c r="O668" t="b">
+        <v>1</v>
+      </c>
+      <c r="P668" t="inlineStr">
+        <is>
+          <t>smp_fpn_r18</t>
+        </is>
+      </c>
+      <c r="Q668" t="n">
+        <v>0.2388743196980337</v>
+      </c>
+      <c r="R668" t="n">
+        <v>0</v>
+      </c>
+      <c r="S668" t="n">
+        <v>0</v>
+      </c>
+      <c r="T668" t="inlineStr">
+        <is>
+          <t>confirmed_holdout</t>
+        </is>
+      </c>
+      <c r="U668" t="inlineStr">
+        <is>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage4_confirmation/facies_f3/metrics.json</t>
+        </is>
+      </c>
+      <c r="V668" t="inlineStr">
+        <is>
+          <t>facies_f3/refit_final.ckpt</t>
+        </is>
+      </c>
+      <c r="W668" t="inlineStr">
+        <is>
+          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+        </is>
+      </c>
+      <c r="X668" t="inlineStr">
+        <is>
+          <t>holdout_confirmation_after_locked_refit</t>
+        </is>
+      </c>
+      <c r="Y668" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z668" t="inlineStr">
+        <is>
+          <t>known holdout confirmed exactly once; no calibration or threshold tuning</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>facies</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>segmentation_2d</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>smp_fpn_r18</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>SMP FPN ResNet18</t>
+        </is>
+      </c>
+      <c r="F669" t="b">
+        <v>0</v>
+      </c>
+      <c r="G669" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="H669" t="inlineStr">
+        <is>
+          <t>refit_final_holdout_confirmation</t>
+        </is>
+      </c>
+      <c r="I669" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J669" t="inlineStr">
+        <is>
+          <t>9a14758fcbf9acd0ab3f8436e923e9fde347e77ce9c42961c113140a9b5407c4</t>
+        </is>
+      </c>
+      <c r="K669" t="inlineStr">
+        <is>
+          <t>p5_stage4_known_holdout</t>
+        </is>
+      </c>
+      <c r="L669" t="inlineStr">
+        <is>
+          <t>refit_final</t>
+        </is>
+      </c>
+      <c r="M669" t="inlineStr">
+        <is>
+          <t>miou</t>
+        </is>
+      </c>
+      <c r="N669" t="n">
+        <v>0.1264948345532109</v>
+      </c>
+      <c r="O669" t="b">
+        <v>1</v>
+      </c>
+      <c r="P669" t="inlineStr">
+        <is>
+          <t>smp_fpn_r18</t>
+        </is>
+      </c>
+      <c r="Q669" t="n">
+        <v>0.1264948345532109</v>
+      </c>
+      <c r="R669" t="n">
+        <v>0</v>
+      </c>
+      <c r="S669" t="n">
+        <v>0</v>
+      </c>
+      <c r="T669" t="inlineStr">
+        <is>
+          <t>confirmed_holdout</t>
+        </is>
+      </c>
+      <c r="U669" t="inlineStr">
+        <is>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage4_confirmation/facies_f3/metrics.json</t>
+        </is>
+      </c>
+      <c r="V669" t="inlineStr">
+        <is>
+          <t>facies_f3/refit_final.ckpt</t>
+        </is>
+      </c>
+      <c r="W669" t="inlineStr">
+        <is>
+          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+        </is>
+      </c>
+      <c r="X669" t="inlineStr">
+        <is>
+          <t>holdout_confirmation_after_locked_refit</t>
+        </is>
+      </c>
+      <c r="Y669" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z669" t="inlineStr">
+        <is>
+          <t>known holdout confirmed exactly once; no calibration or threshold tuning</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>facies</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>segmentation_2d</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>smp_fpn_r18</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>SMP FPN ResNet18</t>
+        </is>
+      </c>
+      <c r="F670" t="b">
+        <v>0</v>
+      </c>
+      <c r="G670" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="H670" t="inlineStr">
+        <is>
+          <t>refit_final_holdout_confirmation</t>
+        </is>
+      </c>
+      <c r="I670" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J670" t="inlineStr">
+        <is>
+          <t>9a14758fcbf9acd0ab3f8436e923e9fde347e77ce9c42961c113140a9b5407c4</t>
+        </is>
+      </c>
+      <c r="K670" t="inlineStr">
+        <is>
+          <t>p5_stage4_known_holdout</t>
+        </is>
+      </c>
+      <c r="L670" t="inlineStr">
+        <is>
+          <t>refit_final</t>
+        </is>
+      </c>
+      <c r="M670" t="inlineStr">
+        <is>
+          <t>macro_f1</t>
+        </is>
+      </c>
+      <c r="N670" t="n">
+        <v>0.2178131390049433</v>
+      </c>
+      <c r="O670" t="b">
+        <v>1</v>
+      </c>
+      <c r="P670" t="inlineStr">
+        <is>
+          <t>smp_fpn_r18</t>
+        </is>
+      </c>
+      <c r="Q670" t="n">
+        <v>0.2178131390049433</v>
+      </c>
+      <c r="R670" t="n">
+        <v>0</v>
+      </c>
+      <c r="S670" t="n">
+        <v>0</v>
+      </c>
+      <c r="T670" t="inlineStr">
+        <is>
+          <t>confirmed_holdout</t>
+        </is>
+      </c>
+      <c r="U670" t="inlineStr">
+        <is>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage4_confirmation/facies_f3/metrics.json</t>
+        </is>
+      </c>
+      <c r="V670" t="inlineStr">
+        <is>
+          <t>facies_f3/refit_final.ckpt</t>
+        </is>
+      </c>
+      <c r="W670" t="inlineStr">
+        <is>
+          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+        </is>
+      </c>
+      <c r="X670" t="inlineStr">
+        <is>
+          <t>holdout_confirmation_after_locked_refit</t>
+        </is>
+      </c>
+      <c r="Y670" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z670" t="inlineStr">
+        <is>
+          <t>known holdout confirmed exactly once; no calibration or threshold tuning</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>facies</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>segmentation_2d</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>smp_fpn_r18</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>SMP FPN ResNet18</t>
+        </is>
+      </c>
+      <c r="F671" t="b">
+        <v>0</v>
+      </c>
+      <c r="G671" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="H671" t="inlineStr">
+        <is>
+          <t>refit_final_holdout_confirmation</t>
+        </is>
+      </c>
+      <c r="I671" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J671" t="inlineStr">
+        <is>
+          <t>9a14758fcbf9acd0ab3f8436e923e9fde347e77ce9c42961c113140a9b5407c4</t>
+        </is>
+      </c>
+      <c r="K671" t="inlineStr">
+        <is>
+          <t>p5_stage4_known_holdout</t>
+        </is>
+      </c>
+      <c r="L671" t="inlineStr">
+        <is>
+          <t>refit_final</t>
+        </is>
+      </c>
+      <c r="M671" t="inlineStr">
+        <is>
+          <t>ece</t>
+        </is>
+      </c>
+      <c r="N671" t="n">
+        <v>0.2519504074355844</v>
+      </c>
+      <c r="O671" t="b">
+        <v>0</v>
+      </c>
+      <c r="P671" t="inlineStr">
+        <is>
+          <t>smp_fpn_r18</t>
+        </is>
+      </c>
+      <c r="Q671" t="n">
+        <v>0.2519504074355844</v>
+      </c>
+      <c r="R671" t="n">
+        <v>0</v>
+      </c>
+      <c r="S671" t="n">
+        <v>0</v>
+      </c>
+      <c r="T671" t="inlineStr">
+        <is>
+          <t>confirmed_holdout</t>
+        </is>
+      </c>
+      <c r="U671" t="inlineStr">
+        <is>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage4_confirmation/facies_f3/metrics.json</t>
+        </is>
+      </c>
+      <c r="V671" t="inlineStr">
+        <is>
+          <t>facies_f3/refit_final.ckpt</t>
+        </is>
+      </c>
+      <c r="W671" t="inlineStr">
+        <is>
+          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+        </is>
+      </c>
+      <c r="X671" t="inlineStr">
+        <is>
+          <t>holdout_confirmation_after_locked_refit</t>
+        </is>
+      </c>
+      <c r="Y671" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z671" t="inlineStr">
+        <is>
+          <t>known holdout confirmed exactly once; no calibration or threshold tuning</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>facies</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>segmentation_2d</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>smp_fpn_r18</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>SMP FPN ResNet18</t>
+        </is>
+      </c>
+      <c r="F672" t="b">
+        <v>0</v>
+      </c>
+      <c r="G672" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="H672" t="inlineStr">
+        <is>
+          <t>refit_final_holdout_confirmation</t>
+        </is>
+      </c>
+      <c r="I672" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J672" t="inlineStr">
+        <is>
+          <t>9a14758fcbf9acd0ab3f8436e923e9fde347e77ce9c42961c113140a9b5407c4</t>
+        </is>
+      </c>
+      <c r="K672" t="inlineStr">
+        <is>
+          <t>p5_stage4_known_holdout</t>
+        </is>
+      </c>
+      <c r="L672" t="inlineStr">
+        <is>
+          <t>refit_final</t>
+        </is>
+      </c>
+      <c r="M672" t="inlineStr">
+        <is>
+          <t>brier</t>
+        </is>
+      </c>
+      <c r="N672" t="n">
+        <v>0.9753594398070996</v>
+      </c>
+      <c r="O672" t="b">
+        <v>0</v>
+      </c>
+      <c r="P672" t="inlineStr">
+        <is>
+          <t>smp_fpn_r18</t>
+        </is>
+      </c>
+      <c r="Q672" t="n">
+        <v>0.9753594398070996</v>
+      </c>
+      <c r="R672" t="n">
+        <v>0</v>
+      </c>
+      <c r="S672" t="n">
+        <v>0</v>
+      </c>
+      <c r="T672" t="inlineStr">
+        <is>
+          <t>confirmed_holdout</t>
+        </is>
+      </c>
+      <c r="U672" t="inlineStr">
+        <is>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage4_confirmation/facies_f3/metrics.json</t>
+        </is>
+      </c>
+      <c r="V672" t="inlineStr">
+        <is>
+          <t>facies_f3/refit_final.ckpt</t>
+        </is>
+      </c>
+      <c r="W672" t="inlineStr">
+        <is>
+          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+        </is>
+      </c>
+      <c r="X672" t="inlineStr">
+        <is>
+          <t>holdout_confirmation_after_locked_refit</t>
+        </is>
+      </c>
+      <c r="Y672" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z672" t="inlineStr">
+        <is>
+          <t>known holdout confirmed exactly once; no calibration or threshold tuning</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>facies</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>segmentation_2d</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>smp_fpn_r18</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>SMP FPN ResNet18</t>
+        </is>
+      </c>
+      <c r="F673" t="b">
+        <v>0</v>
+      </c>
+      <c r="G673" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="H673" t="inlineStr">
+        <is>
+          <t>refit_final_holdout_confirmation</t>
+        </is>
+      </c>
+      <c r="I673" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J673" t="inlineStr">
+        <is>
+          <t>9a14758fcbf9acd0ab3f8436e923e9fde347e77ce9c42961c113140a9b5407c4</t>
+        </is>
+      </c>
+      <c r="K673" t="inlineStr">
+        <is>
+          <t>p5_stage4_known_holdout</t>
+        </is>
+      </c>
+      <c r="L673" t="inlineStr">
+        <is>
+          <t>refit_final</t>
+        </is>
+      </c>
+      <c r="M673" t="inlineStr">
+        <is>
+          <t>nll</t>
+        </is>
+      </c>
+      <c r="N673" t="n">
+        <v>2.874396510552791</v>
+      </c>
+      <c r="O673" t="b">
+        <v>0</v>
+      </c>
+      <c r="P673" t="inlineStr">
+        <is>
+          <t>smp_fpn_r18</t>
+        </is>
+      </c>
+      <c r="Q673" t="n">
+        <v>2.874396510552791</v>
+      </c>
+      <c r="R673" t="n">
+        <v>0</v>
+      </c>
+      <c r="S673" t="n">
+        <v>0</v>
+      </c>
+      <c r="T673" t="inlineStr">
+        <is>
+          <t>confirmed_holdout</t>
+        </is>
+      </c>
+      <c r="U673" t="inlineStr">
+        <is>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage4_confirmation/facies_f3/metrics.json</t>
+        </is>
+      </c>
+      <c r="V673" t="inlineStr">
+        <is>
+          <t>facies_f3/refit_final.ckpt</t>
+        </is>
+      </c>
+      <c r="W673" t="inlineStr">
+        <is>
+          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+        </is>
+      </c>
+      <c r="X673" t="inlineStr">
+        <is>
+          <t>holdout_confirmation_after_locked_refit</t>
+        </is>
+      </c>
+      <c r="Y673" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z673" t="inlineStr">
+        <is>
+          <t>known holdout confirmed exactly once; no calibration or threshold tuning</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>facies</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>Penobscot</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>segmentation_2d</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>smp_deeplabv3plus_r18</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>SMP DeepLabV3+ ResNet18</t>
+        </is>
+      </c>
+      <c r="F674" t="b">
+        <v>0</v>
+      </c>
+      <c r="G674" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="H674" t="inlineStr">
+        <is>
+          <t>refit_final_holdout_confirmation</t>
+        </is>
+      </c>
+      <c r="I674" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J674" t="inlineStr">
+        <is>
+          <t>399a258d1fdc8c396891f2735d7ee95d9d467bf0f43f209e0a0a9213266331e9</t>
+        </is>
+      </c>
+      <c r="K674" t="inlineStr">
+        <is>
+          <t>p5_stage4_known_holdout</t>
+        </is>
+      </c>
+      <c r="L674" t="inlineStr">
+        <is>
+          <t>refit_final</t>
+        </is>
+      </c>
+      <c r="M674" t="inlineStr">
+        <is>
+          <t>accuracy</t>
+        </is>
+      </c>
+      <c r="N674" t="n">
+        <v>0.5285719215618407</v>
+      </c>
+      <c r="O674" t="b">
+        <v>1</v>
+      </c>
+      <c r="P674" t="inlineStr">
+        <is>
+          <t>smp_deeplabv3plus_r18</t>
+        </is>
+      </c>
+      <c r="Q674" t="n">
+        <v>0.5285719215618407</v>
+      </c>
+      <c r="R674" t="n">
+        <v>0</v>
+      </c>
+      <c r="S674" t="n">
+        <v>0</v>
+      </c>
+      <c r="T674" t="inlineStr">
+        <is>
+          <t>confirmed_holdout</t>
+        </is>
+      </c>
+      <c r="U674" t="inlineStr">
+        <is>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage4_confirmation/facies_penobscot/metrics.json</t>
+        </is>
+      </c>
+      <c r="V674" t="inlineStr">
+        <is>
+          <t>facies_penobscot/refit_final.ckpt</t>
+        </is>
+      </c>
+      <c r="W674" t="inlineStr">
+        <is>
+          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+        </is>
+      </c>
+      <c r="X674" t="inlineStr">
+        <is>
+          <t>holdout_confirmation_after_locked_refit</t>
+        </is>
+      </c>
+      <c r="Y674" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z674" t="inlineStr">
+        <is>
+          <t>known holdout confirmed exactly once; no calibration or threshold tuning</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>facies</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>Penobscot</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>segmentation_2d</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>smp_deeplabv3plus_r18</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>SMP DeepLabV3+ ResNet18</t>
+        </is>
+      </c>
+      <c r="F675" t="b">
+        <v>0</v>
+      </c>
+      <c r="G675" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="H675" t="inlineStr">
+        <is>
+          <t>refit_final_holdout_confirmation</t>
+        </is>
+      </c>
+      <c r="I675" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J675" t="inlineStr">
+        <is>
+          <t>399a258d1fdc8c396891f2735d7ee95d9d467bf0f43f209e0a0a9213266331e9</t>
+        </is>
+      </c>
+      <c r="K675" t="inlineStr">
+        <is>
+          <t>p5_stage4_known_holdout</t>
+        </is>
+      </c>
+      <c r="L675" t="inlineStr">
+        <is>
+          <t>refit_final</t>
+        </is>
+      </c>
+      <c r="M675" t="inlineStr">
+        <is>
+          <t>miou</t>
+        </is>
+      </c>
+      <c r="N675" t="n">
+        <v>0.125379989161776</v>
+      </c>
+      <c r="O675" t="b">
+        <v>1</v>
+      </c>
+      <c r="P675" t="inlineStr">
+        <is>
+          <t>smp_deeplabv3plus_r18</t>
+        </is>
+      </c>
+      <c r="Q675" t="n">
+        <v>0.125379989161776</v>
+      </c>
+      <c r="R675" t="n">
+        <v>0</v>
+      </c>
+      <c r="S675" t="n">
+        <v>0</v>
+      </c>
+      <c r="T675" t="inlineStr">
+        <is>
+          <t>confirmed_holdout</t>
+        </is>
+      </c>
+      <c r="U675" t="inlineStr">
+        <is>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage4_confirmation/facies_penobscot/metrics.json</t>
+        </is>
+      </c>
+      <c r="V675" t="inlineStr">
+        <is>
+          <t>facies_penobscot/refit_final.ckpt</t>
+        </is>
+      </c>
+      <c r="W675" t="inlineStr">
+        <is>
+          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+        </is>
+      </c>
+      <c r="X675" t="inlineStr">
+        <is>
+          <t>holdout_confirmation_after_locked_refit</t>
+        </is>
+      </c>
+      <c r="Y675" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z675" t="inlineStr">
+        <is>
+          <t>known holdout confirmed exactly once; no calibration or threshold tuning</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>facies</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>Penobscot</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>segmentation_2d</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>smp_deeplabv3plus_r18</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>SMP DeepLabV3+ ResNet18</t>
+        </is>
+      </c>
+      <c r="F676" t="b">
+        <v>0</v>
+      </c>
+      <c r="G676" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="H676" t="inlineStr">
+        <is>
+          <t>refit_final_holdout_confirmation</t>
+        </is>
+      </c>
+      <c r="I676" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J676" t="inlineStr">
+        <is>
+          <t>399a258d1fdc8c396891f2735d7ee95d9d467bf0f43f209e0a0a9213266331e9</t>
+        </is>
+      </c>
+      <c r="K676" t="inlineStr">
+        <is>
+          <t>p5_stage4_known_holdout</t>
+        </is>
+      </c>
+      <c r="L676" t="inlineStr">
+        <is>
+          <t>refit_final</t>
+        </is>
+      </c>
+      <c r="M676" t="inlineStr">
+        <is>
+          <t>macro_f1</t>
+        </is>
+      </c>
+      <c r="N676" t="n">
+        <v>0.1709165211603197</v>
+      </c>
+      <c r="O676" t="b">
+        <v>1</v>
+      </c>
+      <c r="P676" t="inlineStr">
+        <is>
+          <t>smp_deeplabv3plus_r18</t>
+        </is>
+      </c>
+      <c r="Q676" t="n">
+        <v>0.1709165211603197</v>
+      </c>
+      <c r="R676" t="n">
+        <v>0</v>
+      </c>
+      <c r="S676" t="n">
+        <v>0</v>
+      </c>
+      <c r="T676" t="inlineStr">
+        <is>
+          <t>confirmed_holdout</t>
+        </is>
+      </c>
+      <c r="U676" t="inlineStr">
+        <is>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage4_confirmation/facies_penobscot/metrics.json</t>
+        </is>
+      </c>
+      <c r="V676" t="inlineStr">
+        <is>
+          <t>facies_penobscot/refit_final.ckpt</t>
+        </is>
+      </c>
+      <c r="W676" t="inlineStr">
+        <is>
+          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+        </is>
+      </c>
+      <c r="X676" t="inlineStr">
+        <is>
+          <t>holdout_confirmation_after_locked_refit</t>
+        </is>
+      </c>
+      <c r="Y676" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z676" t="inlineStr">
+        <is>
+          <t>known holdout confirmed exactly once; no calibration or threshold tuning</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>facies</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>Penobscot</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>segmentation_2d</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>smp_deeplabv3plus_r18</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>SMP DeepLabV3+ ResNet18</t>
+        </is>
+      </c>
+      <c r="F677" t="b">
+        <v>0</v>
+      </c>
+      <c r="G677" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="H677" t="inlineStr">
+        <is>
+          <t>refit_final_holdout_confirmation</t>
+        </is>
+      </c>
+      <c r="I677" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J677" t="inlineStr">
+        <is>
+          <t>399a258d1fdc8c396891f2735d7ee95d9d467bf0f43f209e0a0a9213266331e9</t>
+        </is>
+      </c>
+      <c r="K677" t="inlineStr">
+        <is>
+          <t>p5_stage4_known_holdout</t>
+        </is>
+      </c>
+      <c r="L677" t="inlineStr">
+        <is>
+          <t>refit_final</t>
+        </is>
+      </c>
+      <c r="M677" t="inlineStr">
+        <is>
+          <t>ece</t>
+        </is>
+      </c>
+      <c r="N677" t="n">
+        <v>0.2939335861584093</v>
+      </c>
+      <c r="O677" t="b">
+        <v>0</v>
+      </c>
+      <c r="P677" t="inlineStr">
+        <is>
+          <t>smp_deeplabv3plus_r18</t>
+        </is>
+      </c>
+      <c r="Q677" t="n">
+        <v>0.2939335861584093</v>
+      </c>
+      <c r="R677" t="n">
+        <v>0</v>
+      </c>
+      <c r="S677" t="n">
+        <v>0</v>
+      </c>
+      <c r="T677" t="inlineStr">
+        <is>
+          <t>confirmed_holdout</t>
+        </is>
+      </c>
+      <c r="U677" t="inlineStr">
+        <is>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage4_confirmation/facies_penobscot/metrics.json</t>
+        </is>
+      </c>
+      <c r="V677" t="inlineStr">
+        <is>
+          <t>facies_penobscot/refit_final.ckpt</t>
+        </is>
+      </c>
+      <c r="W677" t="inlineStr">
+        <is>
+          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+        </is>
+      </c>
+      <c r="X677" t="inlineStr">
+        <is>
+          <t>holdout_confirmation_after_locked_refit</t>
+        </is>
+      </c>
+      <c r="Y677" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z677" t="inlineStr">
+        <is>
+          <t>known holdout confirmed exactly once; no calibration or threshold tuning</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>facies</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>Penobscot</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>segmentation_2d</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>smp_deeplabv3plus_r18</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>SMP DeepLabV3+ ResNet18</t>
+        </is>
+      </c>
+      <c r="F678" t="b">
+        <v>0</v>
+      </c>
+      <c r="G678" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="H678" t="inlineStr">
+        <is>
+          <t>refit_final_holdout_confirmation</t>
+        </is>
+      </c>
+      <c r="I678" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J678" t="inlineStr">
+        <is>
+          <t>399a258d1fdc8c396891f2735d7ee95d9d467bf0f43f209e0a0a9213266331e9</t>
+        </is>
+      </c>
+      <c r="K678" t="inlineStr">
+        <is>
+          <t>p5_stage4_known_holdout</t>
+        </is>
+      </c>
+      <c r="L678" t="inlineStr">
+        <is>
+          <t>refit_final</t>
+        </is>
+      </c>
+      <c r="M678" t="inlineStr">
+        <is>
+          <t>brier</t>
+        </is>
+      </c>
+      <c r="N678" t="n">
+        <v>0.7475083526250967</v>
+      </c>
+      <c r="O678" t="b">
+        <v>0</v>
+      </c>
+      <c r="P678" t="inlineStr">
+        <is>
+          <t>smp_deeplabv3plus_r18</t>
+        </is>
+      </c>
+      <c r="Q678" t="n">
+        <v>0.7475083526250967</v>
+      </c>
+      <c r="R678" t="n">
+        <v>0</v>
+      </c>
+      <c r="S678" t="n">
+        <v>0</v>
+      </c>
+      <c r="T678" t="inlineStr">
+        <is>
+          <t>confirmed_holdout</t>
+        </is>
+      </c>
+      <c r="U678" t="inlineStr">
+        <is>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage4_confirmation/facies_penobscot/metrics.json</t>
+        </is>
+      </c>
+      <c r="V678" t="inlineStr">
+        <is>
+          <t>facies_penobscot/refit_final.ckpt</t>
+        </is>
+      </c>
+      <c r="W678" t="inlineStr">
+        <is>
+          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+        </is>
+      </c>
+      <c r="X678" t="inlineStr">
+        <is>
+          <t>holdout_confirmation_after_locked_refit</t>
+        </is>
+      </c>
+      <c r="Y678" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z678" t="inlineStr">
+        <is>
+          <t>known holdout confirmed exactly once; no calibration or threshold tuning</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>facies</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>Penobscot</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>segmentation_2d</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>smp_deeplabv3plus_r18</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>SMP DeepLabV3+ ResNet18</t>
+        </is>
+      </c>
+      <c r="F679" t="b">
+        <v>0</v>
+      </c>
+      <c r="G679" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="H679" t="inlineStr">
+        <is>
+          <t>refit_final_holdout_confirmation</t>
+        </is>
+      </c>
+      <c r="I679" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J679" t="inlineStr">
+        <is>
+          <t>399a258d1fdc8c396891f2735d7ee95d9d467bf0f43f209e0a0a9213266331e9</t>
+        </is>
+      </c>
+      <c r="K679" t="inlineStr">
+        <is>
+          <t>p5_stage4_known_holdout</t>
+        </is>
+      </c>
+      <c r="L679" t="inlineStr">
+        <is>
+          <t>refit_final</t>
+        </is>
+      </c>
+      <c r="M679" t="inlineStr">
+        <is>
+          <t>nll</t>
+        </is>
+      </c>
+      <c r="N679" t="n">
+        <v>1.879265954669352</v>
+      </c>
+      <c r="O679" t="b">
+        <v>0</v>
+      </c>
+      <c r="P679" t="inlineStr">
+        <is>
+          <t>smp_deeplabv3plus_r18</t>
+        </is>
+      </c>
+      <c r="Q679" t="n">
+        <v>1.879265954669352</v>
+      </c>
+      <c r="R679" t="n">
+        <v>0</v>
+      </c>
+      <c r="S679" t="n">
+        <v>0</v>
+      </c>
+      <c r="T679" t="inlineStr">
+        <is>
+          <t>confirmed_holdout</t>
+        </is>
+      </c>
+      <c r="U679" t="inlineStr">
+        <is>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage4_confirmation/facies_penobscot/metrics.json</t>
+        </is>
+      </c>
+      <c r="V679" t="inlineStr">
+        <is>
+          <t>facies_penobscot/refit_final.ckpt</t>
+        </is>
+      </c>
+      <c r="W679" t="inlineStr">
+        <is>
+          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+        </is>
+      </c>
+      <c r="X679" t="inlineStr">
+        <is>
+          <t>holdout_confirmation_after_locked_refit</t>
+        </is>
+      </c>
+      <c r="Y679" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z679" t="inlineStr">
+        <is>
+          <t>known holdout confirmed exactly once; no calibration or threshold tuning</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>facies</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>segmentation_2d</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>smp_fpn_r18</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>smp fpn r18</t>
+        </is>
+      </c>
+      <c r="F680" t="b">
+        <v>0</v>
+      </c>
+      <c r="G680" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="H680" t="inlineStr">
+        <is>
+          <t>stage3_oof_leaderboard</t>
+        </is>
+      </c>
+      <c r="I680" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J680" t="inlineStr">
+        <is>
+          <t>d67e14ff951b63551948bd0bf3902ad140672a875e911ad849ba4adae22ac294</t>
+        </is>
+      </c>
+      <c r="K680" t="inlineStr">
+        <is>
+          <t>p5_stage3_oof_aggregate</t>
+        </is>
+      </c>
+      <c r="L680" t="inlineStr">
+        <is>
+          <t>aggregate_oof</t>
+        </is>
+      </c>
+      <c r="M680" t="inlineStr">
+        <is>
+          <t>miou</t>
+        </is>
+      </c>
+      <c r="N680" t="n">
+        <v>0.1313164220202209</v>
+      </c>
+      <c r="O680" t="b">
+        <v>1</v>
+      </c>
+      <c r="P680" t="inlineStr">
+        <is>
+          <t>smp_fpn_r18</t>
+        </is>
+      </c>
+      <c r="Q680" t="n">
+        <v>0.1313164220202209</v>
+      </c>
+      <c r="R680" t="n">
+        <v>0</v>
+      </c>
+      <c r="S680" t="n">
+        <v>0</v>
+      </c>
+      <c r="T680" t="inlineStr">
+        <is>
+          <t>ranked</t>
+        </is>
+      </c>
+      <c r="U680" t="inlineStr">
+        <is>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage3/facies_f3_scratch_leaderboard.json</t>
+        </is>
+      </c>
+      <c r="V680" t="inlineStr"/>
+      <c r="W680" t="inlineStr">
+        <is>
+          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+        </is>
+      </c>
+      <c r="X680" t="inlineStr">
+        <is>
           <t>current_locked_baseline_reference</t>
         </is>
       </c>
-      <c r="Y667" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="Z667" t="inlineStr">
+      <c r="Y680" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z680" t="inlineStr">
+        <is>
+          <t>top-of-board locked baseline from frozen stage-3 leaderboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>facies</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>Penobscot</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>segmentation_2d</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>smp_deeplabv3plus_r18</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>smp deeplabv3plus r18</t>
+        </is>
+      </c>
+      <c r="F681" t="b">
+        <v>0</v>
+      </c>
+      <c r="G681" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="H681" t="inlineStr">
+        <is>
+          <t>stage3_oof_leaderboard</t>
+        </is>
+      </c>
+      <c r="I681" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J681" t="inlineStr">
+        <is>
+          <t>d67e14ff951b63551948bd0bf3902ad140672a875e911ad849ba4adae22ac294</t>
+        </is>
+      </c>
+      <c r="K681" t="inlineStr">
+        <is>
+          <t>p5_stage3_oof_aggregate</t>
+        </is>
+      </c>
+      <c r="L681" t="inlineStr">
+        <is>
+          <t>aggregate_oof</t>
+        </is>
+      </c>
+      <c r="M681" t="inlineStr">
+        <is>
+          <t>miou</t>
+        </is>
+      </c>
+      <c r="N681" t="n">
+        <v>0.1320214117468906</v>
+      </c>
+      <c r="O681" t="b">
+        <v>1</v>
+      </c>
+      <c r="P681" t="inlineStr">
+        <is>
+          <t>smp_deeplabv3plus_r18</t>
+        </is>
+      </c>
+      <c r="Q681" t="n">
+        <v>0.1320214117468906</v>
+      </c>
+      <c r="R681" t="n">
+        <v>0</v>
+      </c>
+      <c r="S681" t="n">
+        <v>0</v>
+      </c>
+      <c r="T681" t="inlineStr">
+        <is>
+          <t>ranked</t>
+        </is>
+      </c>
+      <c r="U681" t="inlineStr">
+        <is>
+          <t>_pipelines/02_task_datasets/facies/_outputs/p5_stage3/facies_penobscot_scratch_leaderboard.json</t>
+        </is>
+      </c>
+      <c r="V681" t="inlineStr"/>
+      <c r="W681" t="inlineStr">
+        <is>
+          <t>e4fd5d8a6371c2b0db6ba2258a41349ec6cfb4f7</t>
+        </is>
+      </c>
+      <c r="X681" t="inlineStr">
+        <is>
+          <t>current_locked_baseline_reference</t>
+        </is>
+      </c>
+      <c r="Y681" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z681" t="inlineStr">
         <is>
           <t>top-of-board locked baseline from frozen stage-3 leaderboard</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z667"/>
+  <autoFilter ref="A1:Z681"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>